<commit_message>
Expand assist specialty cards
</commit_message>
<xml_diff>
--- a/outputs/019f7d3d-0c92-7fc3-ad6b-aa8b1d2aacd1/QOMISO_Game_Tour_Card_Catalog.xlsx
+++ b/outputs/019f7d3d-0c92-7fc3-ad6b-aa8b1d2aacd1/QOMISO_Game_Tour_Card_Catalog.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="Rb62d8d3501f94c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="カード一覧" sheetId="2" r:id="R786bbcc390034c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基本カード" sheetId="3" r:id="Redba876f84d54fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="得意技カード" sheetId="4" r:id="R3d29b34818314801"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汎用勝負手" sheetId="5" r:id="R57e259f554ee43a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固有勝負手" sheetId="6" r:id="Rf116ea8a4ddc4a65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高適性アシスト" sheetId="7" r:id="R35c07ec592a14353"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="役割共通" sheetId="8" r:id="Rcbfc487f8e234048"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="カードルール" sheetId="9" r:id="R109e0d760d7340f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="1" r:id="R9961507418a949d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="カード一覧" sheetId="2" r:id="R51a476cd56a34aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基本カード" sheetId="3" r:id="R183be7ff8aa44407"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="得意技カード" sheetId="4" r:id="Rfb626754cfd945a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汎用勝負手" sheetId="5" r:id="Rbe0711abd8be4ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固有勝負手" sheetId="6" r:id="R56d9f088383246a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="高適性アシスト" sheetId="7" r:id="R59d3c59325e14b1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="役割共通" sheetId="8" r:id="Rd6cc4a305c0e4b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="カードルール" sheetId="9" r:id="Rea8240492df34a80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -347,8 +347,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllCardsTable" displayName="AllCardsTable" ref="A4:L153" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L153"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllCardsTable" displayName="AllCardsTable" ref="A4:L161" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L161"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="分類"/>
     <x:tableColumn id="2" name="No."/>
@@ -388,8 +388,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpecialtyCardsTable" displayName="SpecialtyCardsTable" ref="A4:K38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:K38"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpecialtyCardsTable" displayName="SpecialtyCardsTable" ref="A4:K46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:K46"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="分類"/>
     <x:tableColumn id="2" name="No."/>
@@ -740,8 +740,8 @@
         <x:v>全カード定義</x:v>
       </x:c>
       <x:c r="B5" s="15" t="n">
-        <x:f>COUNTA('カード一覧'!$I$5:$I$153)</x:f>
-        <x:v>149</x:v>
+        <x:f>COUNTA('カード一覧'!$I$5:$I$161)</x:f>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>個人カード</x:v>
@@ -910,7 +910,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="25" t="str">
-        <x:v>固有勝負手50枚、汎用勝負手24枚、高適性アシスト勝負手13枚、共通基本28枚、共通得意技16枚、役割共通22枚を検索できます。</x:v>
+        <x:v>固有勝負手50枚、汎用勝負手24枚、高適性アシスト勝負手13枚、共通基本28枚、共通得意技24枚、役割共通22枚を検索できます。</x:v>
       </x:c>
       <x:c r="B2" s="25"/>
       <x:c r="C2" s="25"/>
@@ -4178,7 +4178,7 @@
       <x:c r="C96" s="38" t="str"/>
       <x:c r="D96" s="38" t="str"/>
       <x:c r="E96" s="38" t="str">
-        <x:v>丘陵エース</x:v>
+        <x:v>平坦アシスト</x:v>
       </x:c>
       <x:c r="F96" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4188,16 +4188,16 @@
       </x:c>
       <x:c r="H96" s="41" t="str"/>
       <x:c r="I96" s="38" t="str">
-        <x:v>丘陵加速</x:v>
+        <x:v>位置取り護衛</x:v>
       </x:c>
       <x:c r="J96" s="38" t="str">
-        <x:v>起伏の変化に合わせて加速し、丘陵区間で集団を絞り込む。</x:v>
+        <x:v>混雑した集団内で進路を確保し、味方エースを前方へ引き上げる。</x:v>
       </x:c>
       <x:c r="K96" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L96" s="38" t="str">
-        <x:v>punch / acceleration</x:v>
+        <x:v>positioning / technique / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="34" customHeight="1">
@@ -4208,7 +4208,7 @@
       <x:c r="C97" s="38" t="str"/>
       <x:c r="D97" s="38" t="str"/>
       <x:c r="E97" s="38" t="str">
-        <x:v>丘陵エース</x:v>
+        <x:v>平坦アシスト</x:v>
       </x:c>
       <x:c r="F97" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4218,16 +4218,16 @@
       </x:c>
       <x:c r="H97" s="41" t="str"/>
       <x:c r="I97" s="38" t="str">
-        <x:v>短坂アタック</x:v>
+        <x:v>ローテーション牽引</x:v>
       </x:c>
       <x:c r="J97" s="38" t="str">
-        <x:v>短い急坂で鋭く仕掛け、ライバルとの小さな差を作る。</x:v>
+        <x:v>味方と先頭交代しながら高速巡航を維持し、エースの消耗を抑える。</x:v>
       </x:c>
       <x:c r="K97" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L97" s="38" t="str">
-        <x:v>punch / fighting</x:v>
+        <x:v>cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="34" customHeight="1">
@@ -4238,7 +4238,7 @@
       <x:c r="C98" s="38" t="str"/>
       <x:c r="D98" s="38" t="str"/>
       <x:c r="E98" s="38" t="str">
-        <x:v>丘陵アシスト</x:v>
+        <x:v>丘陵エース</x:v>
       </x:c>
       <x:c r="F98" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4248,16 +4248,16 @@
       </x:c>
       <x:c r="H98" s="41" t="str"/>
       <x:c r="I98" s="38" t="str">
-        <x:v>丘陵ペース</x:v>
+        <x:v>丘陵加速</x:v>
       </x:c>
       <x:c r="J98" s="38" t="str">
-        <x:v>起伏区間を高い一定速度で牽引し、味方エースの脚を残す。</x:v>
+        <x:v>起伏の変化に合わせて加速し、丘陵区間で集団を絞り込む。</x:v>
       </x:c>
       <x:c r="K98" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L98" s="38" t="str">
-        <x:v>punch / stamina / teamwork</x:v>
+        <x:v>punch / acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="34" customHeight="1">
@@ -4268,7 +4268,7 @@
       <x:c r="C99" s="38" t="str"/>
       <x:c r="D99" s="38" t="str"/>
       <x:c r="E99" s="38" t="str">
-        <x:v>丘陵アシスト</x:v>
+        <x:v>丘陵エース</x:v>
       </x:c>
       <x:c r="F99" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4278,16 +4278,16 @@
       </x:c>
       <x:c r="H99" s="41" t="str"/>
       <x:c r="I99" s="38" t="str">
-        <x:v>仕掛け封じ</x:v>
+        <x:v>短坂アタック</x:v>
       </x:c>
       <x:c r="J99" s="38" t="str">
-        <x:v>丘陵で危険な攻撃を追走し、味方エースに代わって差を消す。</x:v>
+        <x:v>短い急坂で鋭く仕掛け、ライバルとの小さな差を作る。</x:v>
       </x:c>
       <x:c r="K99" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L99" s="38" t="str">
-        <x:v>acceleration / fighting / teamwork</x:v>
+        <x:v>punch / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="34" customHeight="1">
@@ -4298,7 +4298,7 @@
       <x:c r="C100" s="38" t="str"/>
       <x:c r="D100" s="38" t="str"/>
       <x:c r="E100" s="38" t="str">
-        <x:v>山岳エース</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F100" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4308,16 +4308,16 @@
       </x:c>
       <x:c r="H100" s="41" t="str"/>
       <x:c r="I100" s="38" t="str">
-        <x:v>登坂ペースアップ</x:v>
+        <x:v>丘陵ペース</x:v>
       </x:c>
       <x:c r="J100" s="38" t="str">
-        <x:v>登りで段階的に速度を上げ、追走できるライバルを絞り込む。</x:v>
+        <x:v>起伏区間を高い一定速度で牽引し、味方エースの脚を残す。</x:v>
       </x:c>
       <x:c r="K100" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L100" s="38" t="str">
-        <x:v>climbing / stamina</x:v>
+        <x:v>punch / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="34" customHeight="1">
@@ -4328,7 +4328,7 @@
       <x:c r="C101" s="38" t="str"/>
       <x:c r="D101" s="38" t="str"/>
       <x:c r="E101" s="38" t="str">
-        <x:v>山岳エース</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F101" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4338,16 +4338,16 @@
       </x:c>
       <x:c r="H101" s="41" t="str"/>
       <x:c r="I101" s="38" t="str">
-        <x:v>頂上前加速</x:v>
+        <x:v>仕掛け封じ</x:v>
       </x:c>
       <x:c r="J101" s="38" t="str">
-        <x:v>山頂前で加速し、下りへ入る前に有利な位置と時間差を作る。</x:v>
+        <x:v>丘陵で危険な攻撃を追走し、味方エースに代わって差を消す。</x:v>
       </x:c>
       <x:c r="K101" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L101" s="38" t="str">
-        <x:v>climbing / acceleration</x:v>
+        <x:v>acceleration / fighting / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="34" customHeight="1">
@@ -4358,7 +4358,7 @@
       <x:c r="C102" s="38" t="str"/>
       <x:c r="D102" s="38" t="str"/>
       <x:c r="E102" s="38" t="str">
-        <x:v>山岳アシスト</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F102" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4368,16 +4368,16 @@
       </x:c>
       <x:c r="H102" s="41" t="str"/>
       <x:c r="I102" s="38" t="str">
-        <x:v>山岳先導</x:v>
+        <x:v>坂前誘導</x:v>
       </x:c>
       <x:c r="J102" s="38" t="str">
-        <x:v>山岳終盤まで高いペースで牽引し、味方エースを攻撃位置へ運ぶ。</x:v>
+        <x:v>登りに入る前に味方エースを集団前方へ運び、仕掛けへ備える。</x:v>
       </x:c>
       <x:c r="K102" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L102" s="38" t="str">
-        <x:v>climbing / stamina / teamwork</x:v>
+        <x:v>positioning / acceleration / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="34" customHeight="1">
@@ -4388,7 +4388,7 @@
       <x:c r="C103" s="38" t="str"/>
       <x:c r="D103" s="38" t="str"/>
       <x:c r="E103" s="38" t="str">
-        <x:v>山岳アシスト</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F103" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4398,16 +4398,16 @@
       </x:c>
       <x:c r="H103" s="41" t="str"/>
       <x:c r="I103" s="38" t="str">
-        <x:v>登坂チェイス</x:v>
+        <x:v>丘越え牽引</x:v>
       </x:c>
       <x:c r="J103" s="38" t="str">
-        <x:v>登りで生まれた差を一定ペースで詰め、味方エースを先頭へ戻す。</x:v>
+        <x:v>丘の頂上まで牽引し、味方エースの体力と加速力を温存する。</x:v>
       </x:c>
       <x:c r="K103" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L103" s="38" t="str">
-        <x:v>climbing / recovery / teamwork</x:v>
+        <x:v>punch / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="34" customHeight="1">
@@ -4418,7 +4418,7 @@
       <x:c r="C104" s="38" t="str"/>
       <x:c r="D104" s="38" t="str"/>
       <x:c r="E104" s="38" t="str">
-        <x:v>パヴェエース</x:v>
+        <x:v>山岳エース</x:v>
       </x:c>
       <x:c r="F104" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4428,16 +4428,16 @@
       </x:c>
       <x:c r="H104" s="41" t="str"/>
       <x:c r="I104" s="38" t="str">
-        <x:v>石畳加速</x:v>
+        <x:v>登坂ペースアップ</x:v>
       </x:c>
       <x:c r="J104" s="38" t="str">
-        <x:v>安定した走行線から加速し、パヴェ区間で先頭位置を奪う。</x:v>
+        <x:v>登りで段階的に速度を上げ、追走できるライバルを絞り込む。</x:v>
       </x:c>
       <x:c r="K104" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L104" s="38" t="str">
-        <x:v>cobble / acceleration / bike_control</x:v>
+        <x:v>climbing / stamina</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="34" customHeight="1">
@@ -4448,7 +4448,7 @@
       <x:c r="C105" s="38" t="str"/>
       <x:c r="D105" s="38" t="str"/>
       <x:c r="E105" s="38" t="str">
-        <x:v>パヴェエース</x:v>
+        <x:v>山岳エース</x:v>
       </x:c>
       <x:c r="F105" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4458,16 +4458,16 @@
       </x:c>
       <x:c r="H105" s="41" t="str"/>
       <x:c r="I105" s="38" t="str">
-        <x:v>悪路アタック</x:v>
+        <x:v>頂上前加速</x:v>
       </x:c>
       <x:c r="J105" s="38" t="str">
-        <x:v>路面の乱れを利用して仕掛け、悪路に弱いライバルを引き離す。</x:v>
+        <x:v>山頂前で加速し、下りへ入る前に有利な位置と時間差を作る。</x:v>
       </x:c>
       <x:c r="K105" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L105" s="38" t="str">
-        <x:v>cobble / fighting</x:v>
+        <x:v>climbing / acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="34" customHeight="1">
@@ -4478,7 +4478,7 @@
       <x:c r="C106" s="38" t="str"/>
       <x:c r="D106" s="38" t="str"/>
       <x:c r="E106" s="38" t="str">
-        <x:v>パヴェアシスト</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F106" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4488,16 +4488,16 @@
       </x:c>
       <x:c r="H106" s="41" t="str"/>
       <x:c r="I106" s="38" t="str">
-        <x:v>石畳牽引</x:v>
+        <x:v>山岳先導</x:v>
       </x:c>
       <x:c r="J106" s="38" t="str">
-        <x:v>悪路で安全な走行線を保ちながら牽引し、味方エースを前方へ運ぶ。</x:v>
+        <x:v>山岳終盤まで高いペースで牽引し、味方エースを攻撃位置へ運ぶ。</x:v>
       </x:c>
       <x:c r="K106" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L106" s="38" t="str">
-        <x:v>cobble / bike_control / teamwork</x:v>
+        <x:v>climbing / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="34" customHeight="1">
@@ -4508,7 +4508,7 @@
       <x:c r="C107" s="38" t="str"/>
       <x:c r="D107" s="38" t="str"/>
       <x:c r="E107" s="38" t="str">
-        <x:v>パヴェアシスト</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F107" s="38" t="str">
         <x:v>specialty</x:v>
@@ -4518,272 +4518,256 @@
       </x:c>
       <x:c r="H107" s="41" t="str"/>
       <x:c r="I107" s="38" t="str">
-        <x:v>パヴェ追走</x:v>
+        <x:v>登坂チェイス</x:v>
       </x:c>
       <x:c r="J107" s="38" t="str">
-        <x:v>パヴェで先行した危険な選手を追い、味方エースを先頭集団へ戻す。</x:v>
+        <x:v>登りで生まれた差を一定ペースで詰め、味方エースを先頭へ戻す。</x:v>
       </x:c>
       <x:c r="K107" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L107" s="38" t="str">
-        <x:v>cobble / cruise / teamwork</x:v>
+        <x:v>climbing / recovery / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="34" customHeight="1">
       <x:c r="A108" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B108" s="41" t="str"/>
       <x:c r="C108" s="38" t="str"/>
       <x:c r="D108" s="38" t="str"/>
       <x:c r="E108" s="38" t="str">
-        <x:v>平坦エース</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F108" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G108" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H108" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H108" s="41" t="str"/>
       <x:c r="I108" s="38" t="str">
-        <x:v>全開独走</x:v>
+        <x:v>登り口誘導</x:v>
       </x:c>
       <x:c r="J108" s="38" t="str">
-        <x:v>平坦で全力の単独走を開始し、大きなタイム差を狙う。</x:v>
+        <x:v>山岳開始前に集団前方を確保し、味方エースを安全に登りへ入れる。</x:v>
       </x:c>
       <x:c r="K108" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L108" s="38" t="str">
-        <x:v>高速巡航 / 平坦カウンター | cruise / stamina / acceleration</x:v>
+        <x:v>positioning / climbing / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="34" customHeight="1">
       <x:c r="A109" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B109" s="41" t="str"/>
       <x:c r="C109" s="38" t="str"/>
       <x:c r="D109" s="38" t="str"/>
       <x:c r="E109" s="38" t="str">
-        <x:v>平坦エース</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F109" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G109" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H109" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H109" s="41" t="str"/>
       <x:c r="I109" s="38" t="str">
-        <x:v>決定的カウンター</x:v>
+        <x:v>山岳風よけ</x:v>
       </x:c>
       <x:c r="J109" s="38" t="str">
-        <x:v>ライバルの攻撃直後に最大加速し、その動きを逆に勝機へ変える。</x:v>
+        <x:v>登りで風よけとなり、味方エースの体力消費を抑える。</x:v>
       </x:c>
       <x:c r="K109" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L109" s="38" t="str">
-        <x:v>平坦カウンター | acceleration / positioning / fighting</x:v>
+        <x:v>climbing / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="34" customHeight="1">
       <x:c r="A110" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B110" s="41" t="str"/>
       <x:c r="C110" s="38" t="str"/>
       <x:c r="D110" s="38" t="str"/>
       <x:c r="E110" s="38" t="str">
-        <x:v>丘陵エース</x:v>
+        <x:v>パヴェエース</x:v>
       </x:c>
       <x:c r="F110" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G110" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H110" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H110" s="41" t="str"/>
       <x:c r="I110" s="38" t="str">
-        <x:v>丘陵決戦</x:v>
+        <x:v>石畳加速</x:v>
       </x:c>
       <x:c r="J110" s="38" t="str">
-        <x:v>丘陵の勝負所で全力加速し、追走集団を絞り込む。</x:v>
+        <x:v>安定した走行線から加速し、パヴェ区間で先頭位置を奪う。</x:v>
       </x:c>
       <x:c r="K110" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L110" s="38" t="str">
-        <x:v>丘陵加速 / 短坂アタック | punch / acceleration / fighting</x:v>
+        <x:v>cobble / acceleration / bike_control</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="34" customHeight="1">
       <x:c r="A111" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B111" s="41" t="str"/>
       <x:c r="C111" s="38" t="str"/>
       <x:c r="D111" s="38" t="str"/>
       <x:c r="E111" s="38" t="str">
-        <x:v>丘陵エース</x:v>
+        <x:v>パヴェエース</x:v>
       </x:c>
       <x:c r="F111" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G111" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H111" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H111" s="41" t="str"/>
       <x:c r="I111" s="38" t="str">
-        <x:v>短坂決戦</x:v>
+        <x:v>悪路アタック</x:v>
       </x:c>
       <x:c r="J111" s="38" t="str">
-        <x:v>短い急坂へ全力を集中し、頂上までに決定的な差を作る。</x:v>
+        <x:v>路面の乱れを利用して仕掛け、悪路に弱いライバルを引き離す。</x:v>
       </x:c>
       <x:c r="K111" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L111" s="38" t="str">
-        <x:v>短坂アタック | punch / fighting</x:v>
+        <x:v>cobble / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="34" customHeight="1">
       <x:c r="A112" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B112" s="41" t="str"/>
       <x:c r="C112" s="38" t="str"/>
       <x:c r="D112" s="38" t="str"/>
       <x:c r="E112" s="38" t="str">
-        <x:v>山岳エース</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F112" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G112" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H112" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H112" s="41" t="str"/>
       <x:c r="I112" s="38" t="str">
-        <x:v>山岳決戦</x:v>
+        <x:v>石畳牽引</x:v>
       </x:c>
       <x:c r="J112" s="38" t="str">
-        <x:v>長い登りで最大出力を維持し、ライバルを一人ずつ脱落させる。</x:v>
+        <x:v>悪路で安全な走行線を保ちながら牽引し、味方エースを前方へ運ぶ。</x:v>
       </x:c>
       <x:c r="K112" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L112" s="38" t="str">
-        <x:v>登坂ペースアップ / 頂上前加速 | climbing / stamina / fighting</x:v>
+        <x:v>cobble / bike_control / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="34" customHeight="1">
       <x:c r="A113" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B113" s="41" t="str"/>
       <x:c r="C113" s="38" t="str"/>
       <x:c r="D113" s="38" t="str"/>
       <x:c r="E113" s="38" t="str">
-        <x:v>山岳エース</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F113" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G113" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H113" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H113" s="41" t="str"/>
       <x:c r="I113" s="38" t="str">
-        <x:v>頂上前アタック</x:v>
+        <x:v>パヴェ追走</x:v>
       </x:c>
       <x:c r="J113" s="38" t="str">
-        <x:v>山頂前から全力で仕掛け、下りへ入る前に時間差を作る。</x:v>
+        <x:v>パヴェで先行した危険な選手を追い、味方エースを先頭集団へ戻す。</x:v>
       </x:c>
       <x:c r="K113" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L113" s="38" t="str">
-        <x:v>頂上前加速 | climbing / acceleration</x:v>
+        <x:v>cobble / cruise / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="34" customHeight="1">
       <x:c r="A114" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B114" s="41" t="str"/>
       <x:c r="C114" s="38" t="str"/>
       <x:c r="D114" s="38" t="str"/>
       <x:c r="E114" s="38" t="str">
-        <x:v>パヴェエース</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F114" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G114" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H114" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H114" s="41" t="str"/>
       <x:c r="I114" s="38" t="str">
-        <x:v>石畳決戦</x:v>
+        <x:v>石畳進入</x:v>
       </x:c>
       <x:c r="J114" s="38" t="str">
-        <x:v>パヴェで最大加速し、悪路適性の低い選手を脱落させる。</x:v>
+        <x:v>パヴェ区間へ入る前に前方位置を確保し、分断や落車の危険を抑える。</x:v>
       </x:c>
       <x:c r="K114" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L114" s="38" t="str">
-        <x:v>石畳加速 / 悪路アタック | cobble / acceleration / bike_control</x:v>
+        <x:v>positioning / cobble / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="34" customHeight="1">
       <x:c r="A115" s="38" t="str">
-        <x:v>汎用勝負手</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B115" s="41" t="str"/>
       <x:c r="C115" s="38" t="str"/>
       <x:c r="D115" s="38" t="str"/>
       <x:c r="E115" s="38" t="str">
-        <x:v>パヴェエース</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F115" s="38" t="str">
-        <x:v>decisive</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G115" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H115" s="41" t="n">
-        <x:v>1</x:v>
-      </x:c>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H115" s="41" t="str"/>
       <x:c r="I115" s="38" t="str">
-        <x:v>悪路独走</x:v>
+        <x:v>ライン誘導</x:v>
       </x:c>
       <x:c r="J115" s="38" t="str">
-        <x:v>荒れた路面を利用して単独で抜け出し、追走との差を広げる。</x:v>
+        <x:v>石畳で走りやすいラインを示し、味方エースの減速とトラブルを抑える。</x:v>
       </x:c>
       <x:c r="K115" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L115" s="38" t="str">
-        <x:v>悪路アタック | cobble / fighting / stamina</x:v>
+        <x:v>cobble / bike_control / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="34" customHeight="1">
@@ -4794,7 +4778,7 @@
       <x:c r="C116" s="38" t="str"/>
       <x:c r="D116" s="38" t="str"/>
       <x:c r="E116" s="38" t="str">
-        <x:v>逃げエース</x:v>
+        <x:v>平坦エース</x:v>
       </x:c>
       <x:c r="F116" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4806,16 +4790,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I116" s="38" t="str">
-        <x:v>逃げ切り</x:v>
+        <x:v>全開独走</x:v>
       </x:c>
       <x:c r="J116" s="38" t="str">
-        <x:v>残り区間を全力で走り、プロトンの吸収を振り切る。</x:v>
+        <x:v>平坦で全力の単独走を開始し、大きなタイム差を狙う。</x:v>
       </x:c>
       <x:c r="K116" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L116" s="38" t="str">
-        <x:v>逃げ選別 / 逃げ粘り | stamina / cruise / fighting / recovery</x:v>
+        <x:v>高速巡航 / 平坦カウンター | cruise / stamina / acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="34" customHeight="1">
@@ -4826,7 +4810,7 @@
       <x:c r="C117" s="38" t="str"/>
       <x:c r="D117" s="38" t="str"/>
       <x:c r="E117" s="38" t="str">
-        <x:v>逃げエース</x:v>
+        <x:v>平坦エース</x:v>
       </x:c>
       <x:c r="F117" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4838,16 +4822,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I117" s="38" t="str">
-        <x:v>単独ブリッジ</x:v>
+        <x:v>決定的カウンター</x:v>
       </x:c>
       <x:c r="J117" s="38" t="str">
-        <x:v>大きな体力を使って前方集団へ一気に合流する。</x:v>
+        <x:v>ライバルの攻撃直後に最大加速し、その動きを逆に勝機へ変える。</x:v>
       </x:c>
       <x:c r="K117" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L117" s="38" t="str">
-        <x:v>逃げ参加 / ブリッジ | cruise / acceleration / stamina</x:v>
+        <x:v>平坦カウンター | acceleration / positioning / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="34" customHeight="1">
@@ -4858,7 +4842,7 @@
       <x:c r="C118" s="38" t="str"/>
       <x:c r="D118" s="38" t="str"/>
       <x:c r="E118" s="38" t="str">
-        <x:v>下りエース</x:v>
+        <x:v>丘陵エース</x:v>
       </x:c>
       <x:c r="F118" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4870,16 +4854,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I118" s="38" t="str">
-        <x:v>下り勝負</x:v>
+        <x:v>丘陵決戦</x:v>
       </x:c>
       <x:c r="J118" s="38" t="str">
-        <x:v>高速ダウンヒルで仕掛け、後続とのタイム差を広げる。</x:v>
+        <x:v>丘陵の勝負所で全力加速し、追走集団を絞り込む。</x:v>
       </x:c>
       <x:c r="K118" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L118" s="38" t="str">
-        <x:v>下り加速 / 下りアタック | bikeControl / technique / fighting</x:v>
+        <x:v>丘陵加速 / 短坂アタック | punch / acceleration / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="34" customHeight="1">
@@ -4890,7 +4874,7 @@
       <x:c r="C119" s="38" t="str"/>
       <x:c r="D119" s="38" t="str"/>
       <x:c r="E119" s="38" t="str">
-        <x:v>スプリントエース</x:v>
+        <x:v>丘陵エース</x:v>
       </x:c>
       <x:c r="F119" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4902,16 +4886,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I119" s="38" t="str">
-        <x:v>スプリント決戦</x:v>
+        <x:v>短坂決戦</x:v>
       </x:c>
       <x:c r="J119" s="38" t="str">
-        <x:v>フィニッシュへ残した力をすべて使い、最高速で勝負する。</x:v>
+        <x:v>短い急坂へ全力を集中し、頂上までに決定的な差を作る。</x:v>
       </x:c>
       <x:c r="K119" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L119" s="38" t="str">
-        <x:v>高速巡航 / 平坦カウンター | sprint / acceleration / positioning</x:v>
+        <x:v>短坂アタック | punch / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="34" customHeight="1">
@@ -4922,7 +4906,7 @@
       <x:c r="C120" s="38" t="str"/>
       <x:c r="D120" s="38" t="str"/>
       <x:c r="E120" s="38" t="str">
-        <x:v>平坦・TTアシスト</x:v>
+        <x:v>山岳エース</x:v>
       </x:c>
       <x:c r="F120" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4934,16 +4918,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I120" s="38" t="str">
-        <x:v>全開牽引</x:v>
+        <x:v>山岳決戦</x:v>
       </x:c>
       <x:c r="J120" s="38" t="str">
-        <x:v>本人の体力を使い切る高速牽引で、味方エースを勝負区間へ運ぶ。</x:v>
+        <x:v>長い登りで最大出力を維持し、ライバルを一人ずつ脱落させる。</x:v>
       </x:c>
       <x:c r="K120" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L120" s="38" t="str">
-        <x:v>高速牽引 / ハイペース維持 | cruise / stamina / teamwork</x:v>
+        <x:v>登坂ペースアップ / 頂上前加速 | climbing / stamina / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="34" customHeight="1">
@@ -4954,7 +4938,7 @@
       <x:c r="C121" s="38" t="str"/>
       <x:c r="D121" s="38" t="str"/>
       <x:c r="E121" s="38" t="str">
-        <x:v>横風アシスト</x:v>
+        <x:v>山岳エース</x:v>
       </x:c>
       <x:c r="F121" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4966,16 +4950,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I121" s="38" t="str">
-        <x:v>横風防衛</x:v>
+        <x:v>頂上前アタック</x:v>
       </x:c>
       <x:c r="J121" s="38" t="str">
-        <x:v>横風による味方エースの消耗と分断を一度だけ防ぐ。</x:v>
+        <x:v>山頂前から全力で仕掛け、下りへ入る前に時間差を作る。</x:v>
       </x:c>
       <x:c r="K121" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L121" s="38" t="str">
-        <x:v>横風ガード | cruise / positioning / teamwork</x:v>
+        <x:v>頂上前加速 | climbing / acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="34" customHeight="1">
@@ -4986,7 +4970,7 @@
       <x:c r="C122" s="38" t="str"/>
       <x:c r="D122" s="38" t="str"/>
       <x:c r="E122" s="38" t="str">
-        <x:v>丘陵アシスト</x:v>
+        <x:v>パヴェエース</x:v>
       </x:c>
       <x:c r="F122" s="38" t="str">
         <x:v>decisive</x:v>
@@ -4998,16 +4982,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I122" s="38" t="str">
-        <x:v>丘陵封鎖</x:v>
+        <x:v>石畳決戦</x:v>
       </x:c>
       <x:c r="J122" s="38" t="str">
-        <x:v>丘陵で高いペースを維持し、ライバルの攻撃を封じる。</x:v>
+        <x:v>パヴェで最大加速し、悪路適性の低い選手を脱落させる。</x:v>
       </x:c>
       <x:c r="K122" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L122" s="38" t="str">
-        <x:v>丘陵ペース / 仕掛け封じ | punch / stamina / teamwork</x:v>
+        <x:v>石畳加速 / 悪路アタック | cobble / acceleration / bike_control</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="34" customHeight="1">
@@ -5018,7 +5002,7 @@
       <x:c r="C123" s="38" t="str"/>
       <x:c r="D123" s="38" t="str"/>
       <x:c r="E123" s="38" t="str">
-        <x:v>山岳アシスト</x:v>
+        <x:v>パヴェエース</x:v>
       </x:c>
       <x:c r="F123" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5030,16 +5014,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I123" s="38" t="str">
-        <x:v>全力献身</x:v>
+        <x:v>悪路独走</x:v>
       </x:c>
       <x:c r="J123" s="38" t="str">
-        <x:v>山岳で体力を使い切り、味方エースを攻撃位置へ送り出す。</x:v>
+        <x:v>荒れた路面を利用して単独で抜け出し、追走との差を広げる。</x:v>
       </x:c>
       <x:c r="K123" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L123" s="38" t="str">
-        <x:v>山岳先導 / 最後の山岳牽引 | climbing / stamina / recovery / teamwork</x:v>
+        <x:v>悪路アタック | cobble / fighting / stamina</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="34" customHeight="1">
@@ -5050,7 +5034,7 @@
       <x:c r="C124" s="38" t="str"/>
       <x:c r="D124" s="38" t="str"/>
       <x:c r="E124" s="38" t="str">
-        <x:v>山岳アシスト</x:v>
+        <x:v>逃げエース</x:v>
       </x:c>
       <x:c r="F124" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5062,16 +5046,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I124" s="38" t="str">
-        <x:v>山岳救援</x:v>
+        <x:v>逃げ切り</x:v>
       </x:c>
       <x:c r="J124" s="38" t="str">
-        <x:v>山岳で遅れた味方エースを牽引し、先頭集団へ戻す。</x:v>
+        <x:v>残り区間を全力で走り、プロトンの吸収を振り切る。</x:v>
       </x:c>
       <x:c r="K124" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L124" s="38" t="str">
-        <x:v>登坂チェイス / 山岳ペースアップ | climbing / recovery / teamwork</x:v>
+        <x:v>逃げ選別 / 逃げ粘り | stamina / cruise / fighting / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="34" customHeight="1">
@@ -5082,7 +5066,7 @@
       <x:c r="C125" s="38" t="str"/>
       <x:c r="D125" s="38" t="str"/>
       <x:c r="E125" s="38" t="str">
-        <x:v>パヴェアシスト</x:v>
+        <x:v>逃げエース</x:v>
       </x:c>
       <x:c r="F125" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5094,16 +5078,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I125" s="38" t="str">
-        <x:v>石畳護衛</x:v>
+        <x:v>単独ブリッジ</x:v>
       </x:c>
       <x:c r="J125" s="38" t="str">
-        <x:v>パヴェで進路を確保し、味方エースを前方集団へ残す。</x:v>
+        <x:v>大きな体力を使って前方集団へ一気に合流する。</x:v>
       </x:c>
       <x:c r="K125" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L125" s="38" t="str">
-        <x:v>石畳牽引 / パヴェ追走 | cobble / bike_control / teamwork</x:v>
+        <x:v>逃げ参加 / ブリッジ | cruise / acceleration / stamina</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="34" customHeight="1">
@@ -5114,7 +5098,7 @@
       <x:c r="C126" s="38" t="str"/>
       <x:c r="D126" s="38" t="str"/>
       <x:c r="E126" s="38" t="str">
-        <x:v>リードアウト</x:v>
+        <x:v>下りエース</x:v>
       </x:c>
       <x:c r="F126" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5126,16 +5110,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I126" s="38" t="str">
-        <x:v>最終発射</x:v>
+        <x:v>下り勝負</x:v>
       </x:c>
       <x:c r="J126" s="38" t="str">
-        <x:v>味方エースを最高速度でスプリントへ送り出す。</x:v>
+        <x:v>高速ダウンヒルで仕掛け、後続とのタイム差を広げる。</x:v>
       </x:c>
       <x:c r="K126" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L126" s="38" t="str">
-        <x:v>高速リードアウト / トレイン加速 | sprint / acceleration / teamwork</x:v>
+        <x:v>下り加速 / 下りアタック | bikeControl / technique / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="34" customHeight="1">
@@ -5146,7 +5130,7 @@
       <x:c r="C127" s="38" t="str"/>
       <x:c r="D127" s="38" t="str"/>
       <x:c r="E127" s="38" t="str">
-        <x:v>ロードキャプテン</x:v>
+        <x:v>スプリントエース</x:v>
       </x:c>
       <x:c r="F127" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5158,16 +5142,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I127" s="38" t="str">
-        <x:v>緊急再編</x:v>
+        <x:v>スプリント決戦</x:v>
       </x:c>
       <x:c r="J127" s="38" t="str">
-        <x:v>崩れたチーム隊列を即座に組み直し、勝負位置へ戻す。</x:v>
+        <x:v>フィニッシュへ残した力をすべて使い、最高速で勝負する。</x:v>
       </x:c>
       <x:c r="K127" s="38" t="str">
-        <x:v>味方チーム</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="L127" s="38" t="str">
-        <x:v>隊列再編 | teamwork / technique / recovery</x:v>
+        <x:v>高速巡航 / 平坦カウンター | sprint / acceleration / positioning</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="34" customHeight="1">
@@ -5178,7 +5162,7 @@
       <x:c r="C128" s="38" t="str"/>
       <x:c r="D128" s="38" t="str"/>
       <x:c r="E128" s="38" t="str">
-        <x:v>復帰アシスト</x:v>
+        <x:v>平坦・TTアシスト</x:v>
       </x:c>
       <x:c r="F128" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5190,16 +5174,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I128" s="38" t="str">
-        <x:v>全力復帰</x:v>
+        <x:v>全開牽引</x:v>
       </x:c>
       <x:c r="J128" s="38" t="str">
-        <x:v>遅れた味方エースを全力でプロトンへ復帰させる。</x:v>
+        <x:v>本人の体力を使い切る高速牽引で、味方エースを勝負区間へ運ぶ。</x:v>
       </x:c>
       <x:c r="K128" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L128" s="38" t="str">
-        <x:v>集団復帰 / 下り復帰 | cruise / stamina / teamwork</x:v>
+        <x:v>高速牽引 / ハイペース維持 | cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="34" customHeight="1">
@@ -5210,7 +5194,7 @@
       <x:c r="C129" s="38" t="str"/>
       <x:c r="D129" s="38" t="str"/>
       <x:c r="E129" s="38" t="str">
-        <x:v>下りアシスト</x:v>
+        <x:v>横風アシスト</x:v>
       </x:c>
       <x:c r="F129" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5222,16 +5206,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I129" s="38" t="str">
-        <x:v>下り護衛</x:v>
+        <x:v>横風防衛</x:v>
       </x:c>
       <x:c r="J129" s="38" t="str">
-        <x:v>下りで味方エースを安全かつ高速に前方集団へ運ぶ。</x:v>
+        <x:v>横風による味方エースの消耗と分断を一度だけ防ぐ。</x:v>
       </x:c>
       <x:c r="K129" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L129" s="38" t="str">
-        <x:v>ダウンヒル牽引 | bikeControl / technique / teamwork</x:v>
+        <x:v>横風ガード | cruise / positioning / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="34" customHeight="1">
@@ -5242,7 +5226,7 @@
       <x:c r="C130" s="38" t="str"/>
       <x:c r="D130" s="38" t="str"/>
       <x:c r="E130" s="38" t="str">
-        <x:v>プロトンコントロール</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F130" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5254,16 +5238,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I130" s="38" t="str">
-        <x:v>完全吸収</x:v>
+        <x:v>丘陵封鎖</x:v>
       </x:c>
       <x:c r="J130" s="38" t="str">
-        <x:v>チームを全力追走させ、危険な逃げをプロトンへ吸収する。</x:v>
+        <x:v>丘陵で高いペースを維持し、ライバルの攻撃を封じる。</x:v>
       </x:c>
       <x:c r="K130" s="38" t="str">
-        <x:v>味方チーム</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L130" s="38" t="str">
-        <x:v>逃げ吸収 / ハイペース維持 | cruise / stamina / teamwork</x:v>
+        <x:v>丘陵ペース / 仕掛け封じ | punch / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="34" customHeight="1">
@@ -5274,7 +5258,7 @@
       <x:c r="C131" s="38" t="str"/>
       <x:c r="D131" s="38" t="str"/>
       <x:c r="E131" s="38" t="str">
-        <x:v>サテライトアシスト</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F131" s="38" t="str">
         <x:v>decisive</x:v>
@@ -5286,81 +5270,85 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I131" s="38" t="str">
-        <x:v>サテライト救援</x:v>
+        <x:v>全力献身</x:v>
       </x:c>
       <x:c r="J131" s="38" t="str">
-        <x:v>前方待機から合流し、補給・牽引・風よけをまとめて行う。</x:v>
+        <x:v>山岳で体力を使い切り、味方エースを攻撃位置へ送り出す。</x:v>
       </x:c>
       <x:c r="K131" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L131" s="38" t="str">
-        <x:v>サテライト合流 / ブリッジ | climbing / stamina / recovery / teamwork</x:v>
+        <x:v>山岳先導 / 最後の山岳牽引 | climbing / stamina / recovery / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="34" customHeight="1">
       <x:c r="A132" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B132" s="41" t="str"/>
       <x:c r="C132" s="38" t="str"/>
       <x:c r="D132" s="38" t="str"/>
       <x:c r="E132" s="38" t="str">
-        <x:v>サブエース</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F132" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G132" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H132" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H132" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I132" s="38" t="str">
-        <x:v>プランB</x:v>
+        <x:v>山岳救援</x:v>
       </x:c>
       <x:c r="J132" s="38" t="str">
-        <x:v>エースの不調や脱落時に第二の勝利プランへ移行する。</x:v>
+        <x:v>山岳で遅れた味方エースを牽引し、先頭集団へ戻す。</x:v>
       </x:c>
       <x:c r="K132" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L132" s="38" t="str">
-        <x:v>ace_aptitude / recovery / fighting</x:v>
+        <x:v>登坂チェイス / 山岳ペースアップ | climbing / recovery / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="34" customHeight="1">
       <x:c r="A133" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B133" s="41" t="str"/>
       <x:c r="C133" s="38" t="str"/>
       <x:c r="D133" s="38" t="str"/>
       <x:c r="E133" s="38" t="str">
-        <x:v>ロードキャプテン</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F133" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G133" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H133" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H133" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I133" s="38" t="str">
-        <x:v>隊列再編</x:v>
+        <x:v>石畳護衛</x:v>
       </x:c>
       <x:c r="J133" s="38" t="str">
-        <x:v>味方の位置取りと戦術判断を安定させる。</x:v>
+        <x:v>パヴェで進路を確保し、味方エースを前方集団へ残す。</x:v>
       </x:c>
       <x:c r="K133" s="38" t="str">
-        <x:v>味方チーム</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L133" s="38" t="str">
-        <x:v>teamwork / technique / recovery</x:v>
+        <x:v>石畳牽引 / パヴェ追走 | cobble / bike_control / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="34" customHeight="1">
       <x:c r="A134" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B134" s="41" t="str"/>
       <x:c r="C134" s="38" t="str"/>
@@ -5369,173 +5357,185 @@
         <x:v>リードアウト</x:v>
       </x:c>
       <x:c r="F134" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G134" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H134" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H134" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I134" s="38" t="str">
-        <x:v>高速リードアウト</x:v>
+        <x:v>最終発射</x:v>
       </x:c>
       <x:c r="J134" s="38" t="str">
-        <x:v>味方スプリンターの位置取りと加速移行を補助する。</x:v>
+        <x:v>味方エースを最高速度でスプリントへ送り出す。</x:v>
       </x:c>
       <x:c r="K134" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L134" s="38" t="str">
-        <x:v>acceleration / sprint / cruise / teamwork</x:v>
+        <x:v>高速リードアウト / トレイン加速 | sprint / acceleration / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="34" customHeight="1">
       <x:c r="A135" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B135" s="41" t="str"/>
       <x:c r="C135" s="38" t="str"/>
       <x:c r="D135" s="38" t="str"/>
       <x:c r="E135" s="38" t="str">
-        <x:v>スプリントトレイン</x:v>
+        <x:v>ロードキャプテン</x:v>
       </x:c>
       <x:c r="F135" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G135" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H135" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H135" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I135" s="38" t="str">
-        <x:v>トレイン加速</x:v>
+        <x:v>緊急再編</x:v>
       </x:c>
       <x:c r="J135" s="38" t="str">
-        <x:v>終盤の隊列維持と速度の受け渡しを安定させる。</x:v>
+        <x:v>崩れたチーム隊列を即座に組み直し、勝負位置へ戻す。</x:v>
       </x:c>
       <x:c r="K135" s="38" t="str">
         <x:v>味方チーム</x:v>
       </x:c>
       <x:c r="L135" s="38" t="str">
-        <x:v>cruise / acceleration / sprint / teamwork</x:v>
+        <x:v>隊列再編 | teamwork / technique / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="34" customHeight="1">
       <x:c r="A136" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B136" s="41" t="str"/>
       <x:c r="C136" s="38" t="str"/>
       <x:c r="D136" s="38" t="str"/>
       <x:c r="E136" s="38" t="str">
-        <x:v>平坦ペースメーカー</x:v>
+        <x:v>復帰アシスト</x:v>
       </x:c>
       <x:c r="F136" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G136" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H136" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H136" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I136" s="38" t="str">
-        <x:v>ハイペース維持</x:v>
+        <x:v>全力復帰</x:v>
       </x:c>
       <x:c r="J136" s="38" t="str">
-        <x:v>逃げとの差と集団速度を安定させる。</x:v>
+        <x:v>遅れた味方エースを全力でプロトンへ復帰させる。</x:v>
       </x:c>
       <x:c r="K136" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L136" s="38" t="str">
-        <x:v>cruise / stamina / recovery</x:v>
+        <x:v>集団復帰 / 下り復帰 | cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="34" customHeight="1">
       <x:c r="A137" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B137" s="41" t="str"/>
       <x:c r="C137" s="38" t="str"/>
       <x:c r="D137" s="38" t="str"/>
       <x:c r="E137" s="38" t="str">
-        <x:v>山岳番手</x:v>
+        <x:v>下りアシスト</x:v>
       </x:c>
       <x:c r="F137" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G137" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H137" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H137" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I137" s="38" t="str">
-        <x:v>最後の山岳牽引</x:v>
+        <x:v>下り護衛</x:v>
       </x:c>
       <x:c r="J137" s="38" t="str">
-        <x:v>山頂付近の攻撃対応と最終発射を支援する。</x:v>
+        <x:v>下りで味方エースを安全かつ高速に前方集団へ運ぶ。</x:v>
       </x:c>
       <x:c r="K137" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L137" s="38" t="str">
-        <x:v>climb / acceleration / stamina / recovery</x:v>
+        <x:v>ダウンヒル牽引 | bikeControl / technique / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="34" customHeight="1">
       <x:c r="A138" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B138" s="41" t="str"/>
       <x:c r="C138" s="38" t="str"/>
       <x:c r="D138" s="38" t="str"/>
       <x:c r="E138" s="38" t="str">
-        <x:v>山岳ペースメーカー</x:v>
+        <x:v>プロトンコントロール</x:v>
       </x:c>
       <x:c r="F138" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G138" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H138" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H138" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I138" s="38" t="str">
-        <x:v>山岳ペースアップ</x:v>
+        <x:v>完全吸収</x:v>
       </x:c>
       <x:c r="J138" s="38" t="str">
-        <x:v>集団を絞り込み急なアタックを抑制する。</x:v>
+        <x:v>チームを全力追走させ、危険な逃げをプロトンへ吸収する。</x:v>
       </x:c>
       <x:c r="K138" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>味方チーム</x:v>
       </x:c>
       <x:c r="L138" s="38" t="str">
-        <x:v>climb / stamina / cruise</x:v>
+        <x:v>逃げ吸収 / ハイペース維持 | cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="34" customHeight="1">
       <x:c r="A139" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>汎用勝負手</x:v>
       </x:c>
       <x:c r="B139" s="41" t="str"/>
       <x:c r="C139" s="38" t="str"/>
       <x:c r="D139" s="38" t="str"/>
       <x:c r="E139" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>サテライトアシスト</x:v>
       </x:c>
       <x:c r="F139" s="38" t="str">
-        <x:v>specialty</x:v>
+        <x:v>decisive</x:v>
       </x:c>
       <x:c r="G139" s="41" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="H139" s="41" t="str"/>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H139" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I139" s="38" t="str">
-        <x:v>ダウンヒル牽引</x:v>
+        <x:v>サテライト救援</x:v>
       </x:c>
       <x:c r="J139" s="38" t="str">
-        <x:v>下り速度と隊列安定性を高める。</x:v>
+        <x:v>前方待機から合流し、補給・牽引・風よけをまとめて行う。</x:v>
       </x:c>
       <x:c r="K139" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L139" s="38" t="str">
-        <x:v>bikeControl / technique / fighting</x:v>
+        <x:v>サテライト合流 / ブリッジ | climbing / stamina / recovery / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="34" customHeight="1">
@@ -5546,7 +5546,7 @@
       <x:c r="C140" s="38" t="str"/>
       <x:c r="D140" s="38" t="str"/>
       <x:c r="E140" s="38" t="str">
-        <x:v>ブレイクアウェイキラー</x:v>
+        <x:v>サブエース</x:v>
       </x:c>
       <x:c r="F140" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5556,16 +5556,16 @@
       </x:c>
       <x:c r="H140" s="41" t="str"/>
       <x:c r="I140" s="38" t="str">
-        <x:v>逃げ吸収</x:v>
+        <x:v>プランB</x:v>
       </x:c>
       <x:c r="J140" s="38" t="str">
-        <x:v>逃げとのタイム差を効率よく削る。</x:v>
+        <x:v>エースの不調や脱落時に第二の勝利プランへ移行する。</x:v>
       </x:c>
       <x:c r="K140" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L140" s="38" t="str">
-        <x:v>cruise / stamina / teamwork</x:v>
+        <x:v>ace_aptitude / recovery / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="34" customHeight="1">
@@ -5576,7 +5576,7 @@
       <x:c r="C141" s="38" t="str"/>
       <x:c r="D141" s="38" t="str"/>
       <x:c r="E141" s="38" t="str">
-        <x:v>トラブル復帰牽引</x:v>
+        <x:v>ロードキャプテン</x:v>
       </x:c>
       <x:c r="F141" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5586,16 +5586,16 @@
       </x:c>
       <x:c r="H141" s="41" t="str"/>
       <x:c r="I141" s="38" t="str">
-        <x:v>集団復帰</x:v>
+        <x:v>隊列再編</x:v>
       </x:c>
       <x:c r="J141" s="38" t="str">
-        <x:v>復帰速度を上げエースの消耗を抑える。</x:v>
+        <x:v>味方の位置取りと戦術判断を安定させる。</x:v>
       </x:c>
       <x:c r="K141" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>味方チーム</x:v>
       </x:c>
       <x:c r="L141" s="38" t="str">
-        <x:v>cruise / stamina / teamwork</x:v>
+        <x:v>teamwork / technique / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="34" customHeight="1">
@@ -5606,7 +5606,7 @@
       <x:c r="C142" s="38" t="str"/>
       <x:c r="D142" s="38" t="str"/>
       <x:c r="E142" s="38" t="str">
-        <x:v>サテライトライダー</x:v>
+        <x:v>リードアウト</x:v>
       </x:c>
       <x:c r="F142" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5616,16 +5616,16 @@
       </x:c>
       <x:c r="H142" s="41" t="str"/>
       <x:c r="I142" s="38" t="str">
-        <x:v>サテライト合流</x:v>
+        <x:v>高速リードアウト</x:v>
       </x:c>
       <x:c r="J142" s="38" t="str">
-        <x:v>合流後に補給、牽引、風よけを提供する。</x:v>
+        <x:v>味方スプリンターの位置取りと加速移行を補助する。</x:v>
       </x:c>
       <x:c r="K142" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L142" s="38" t="str">
-        <x:v>climb / stamina / recovery / teamwork</x:v>
+        <x:v>acceleration / sprint / cruise / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="34" customHeight="1">
@@ -5636,7 +5636,7 @@
       <x:c r="C143" s="38" t="str"/>
       <x:c r="D143" s="38" t="str"/>
       <x:c r="E143" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>スプリントトレイン</x:v>
       </x:c>
       <x:c r="F143" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5646,16 +5646,16 @@
       </x:c>
       <x:c r="H143" s="41" t="str"/>
       <x:c r="I143" s="38" t="str">
-        <x:v>逃げ参加</x:v>
+        <x:v>トレイン加速</x:v>
       </x:c>
       <x:c r="J143" s="38" t="str">
-        <x:v>序盤の逃げ形成時、逃げ集団へ入る成功率を上げる。</x:v>
+        <x:v>終盤の隊列維持と速度の受け渡しを安定させる。</x:v>
       </x:c>
       <x:c r="K143" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方チーム</x:v>
       </x:c>
       <x:c r="L143" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>cruise / acceleration / sprint / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="34" customHeight="1">
@@ -5666,7 +5666,7 @@
       <x:c r="C144" s="38" t="str"/>
       <x:c r="D144" s="38" t="str"/>
       <x:c r="E144" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>平坦ペースメーカー</x:v>
       </x:c>
       <x:c r="F144" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5676,16 +5676,16 @@
       </x:c>
       <x:c r="H144" s="41" t="str"/>
       <x:c r="I144" s="38" t="str">
-        <x:v>ブリッジ</x:v>
+        <x:v>ハイペース維持</x:v>
       </x:c>
       <x:c r="J144" s="38" t="str">
-        <x:v>メイン集団から加速し、すでに形成された逃げ集団へ合流する。</x:v>
+        <x:v>逃げとの差と集団速度を安定させる。</x:v>
       </x:c>
       <x:c r="K144" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L144" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>cruise / stamina / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="34" customHeight="1">
@@ -5696,26 +5696,26 @@
       <x:c r="C145" s="38" t="str"/>
       <x:c r="D145" s="38" t="str"/>
       <x:c r="E145" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>山岳番手</x:v>
       </x:c>
       <x:c r="F145" s="38" t="str">
-        <x:v>basic</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G145" s="41" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H145" s="41" t="str"/>
       <x:c r="I145" s="38" t="str">
-        <x:v>先頭交代</x:v>
+        <x:v>最後の山岳牽引</x:v>
       </x:c>
       <x:c r="J145" s="38" t="str">
-        <x:v>逃げ集団の先頭を長く引き、本人の体力を使ってタイム差を広げる。</x:v>
+        <x:v>山頂付近の攻撃対応と最終発射を支援する。</x:v>
       </x:c>
       <x:c r="K145" s="38" t="str">
-        <x:v>逃げ集団</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L145" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>climb / acceleration / stamina / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="34" customHeight="1">
@@ -5726,26 +5726,26 @@
       <x:c r="C146" s="38" t="str"/>
       <x:c r="D146" s="38" t="str"/>
       <x:c r="E146" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>山岳ペースメーカー</x:v>
       </x:c>
       <x:c r="F146" s="38" t="str">
-        <x:v>basic</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G146" s="41" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H146" s="41" t="str"/>
       <x:c r="I146" s="38" t="str">
-        <x:v>ペース調整</x:v>
+        <x:v>山岳ペースアップ</x:v>
       </x:c>
       <x:c r="J146" s="38" t="str">
-        <x:v>余計な体力消費を抑えながら、逃げ集団の速度とタイム差を維持する。</x:v>
+        <x:v>集団を絞り込み急なアタックを抑制する。</x:v>
       </x:c>
       <x:c r="K146" s="38" t="str">
-        <x:v>逃げ集団</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L146" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>climb / stamina / cruise</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="34" customHeight="1">
@@ -5756,7 +5756,7 @@
       <x:c r="C147" s="38" t="str"/>
       <x:c r="D147" s="38" t="str"/>
       <x:c r="E147" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>下り牽引</x:v>
       </x:c>
       <x:c r="F147" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5766,16 +5766,16 @@
       </x:c>
       <x:c r="H147" s="41" t="str"/>
       <x:c r="I147" s="38" t="str">
-        <x:v>逃げ選別</x:v>
+        <x:v>ダウンヒル牽引</x:v>
       </x:c>
       <x:c r="J147" s="38" t="str">
-        <x:v>起伏や横風でペースを上げ、逃げ集団の人数を絞り込む。</x:v>
+        <x:v>下り速度と隊列安定性を高める。</x:v>
       </x:c>
       <x:c r="K147" s="38" t="str">
-        <x:v>逃げ集団</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L147" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>bikeControl / technique / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="148" ht="34" customHeight="1">
@@ -5786,7 +5786,7 @@
       <x:c r="C148" s="38" t="str"/>
       <x:c r="D148" s="38" t="str"/>
       <x:c r="E148" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>ブレイクアウェイキラー</x:v>
       </x:c>
       <x:c r="F148" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5796,16 +5796,16 @@
       </x:c>
       <x:c r="H148" s="41" t="str"/>
       <x:c r="I148" s="38" t="str">
-        <x:v>逃げ粘り</x:v>
+        <x:v>逃げ吸収</x:v>
       </x:c>
       <x:c r="J148" s="38" t="str">
-        <x:v>吸収されそうな場面で再加速し、逃げ集団の生存時間を延ばす。</x:v>
+        <x:v>逃げとのタイム差を効率よく削る。</x:v>
       </x:c>
       <x:c r="K148" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L148" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="34" customHeight="1">
@@ -5816,26 +5816,26 @@
       <x:c r="C149" s="38" t="str"/>
       <x:c r="D149" s="38" t="str"/>
       <x:c r="E149" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>トラブル復帰牽引</x:v>
       </x:c>
       <x:c r="F149" s="38" t="str">
-        <x:v>basic</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G149" s="41" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H149" s="41" t="str"/>
       <x:c r="I149" s="38" t="str">
-        <x:v>高速コーナリング</x:v>
+        <x:v>集団復帰</x:v>
       </x:c>
       <x:c r="J149" s="38" t="str">
-        <x:v>コーナーでの速度低下と落車リスクを抑える。</x:v>
+        <x:v>復帰速度を上げエースの消耗を抑える。</x:v>
       </x:c>
       <x:c r="K149" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L149" s="38" t="str">
-        <x:v>bikeControl / technique / fighting</x:v>
+        <x:v>cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="34" customHeight="1">
@@ -5846,7 +5846,7 @@
       <x:c r="C150" s="38" t="str"/>
       <x:c r="D150" s="38" t="str"/>
       <x:c r="E150" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>サテライトライダー</x:v>
       </x:c>
       <x:c r="F150" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5856,16 +5856,16 @@
       </x:c>
       <x:c r="H150" s="41" t="str"/>
       <x:c r="I150" s="38" t="str">
-        <x:v>下り加速</x:v>
+        <x:v>サテライト合流</x:v>
       </x:c>
       <x:c r="J150" s="38" t="str">
-        <x:v>下りの直線で速度を上げ、前方集団との差を縮める。</x:v>
+        <x:v>合流後に補給、牽引、風よけを提供する。</x:v>
       </x:c>
       <x:c r="K150" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="L150" s="38" t="str">
-        <x:v>bikeControl / technique / fighting</x:v>
+        <x:v>climb / stamina / recovery / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="34" customHeight="1">
@@ -5876,7 +5876,7 @@
       <x:c r="C151" s="38" t="str"/>
       <x:c r="D151" s="38" t="str"/>
       <x:c r="E151" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>逃げ屋</x:v>
       </x:c>
       <x:c r="F151" s="38" t="str">
         <x:v>specialty</x:v>
@@ -5886,16 +5886,16 @@
       </x:c>
       <x:c r="H151" s="41" t="str"/>
       <x:c r="I151" s="38" t="str">
-        <x:v>下りアタック</x:v>
+        <x:v>逃げ参加</x:v>
       </x:c>
       <x:c r="J151" s="38" t="str">
-        <x:v>テクニカルな下りで仕掛け、後続とのタイム差を作る。</x:v>
+        <x:v>序盤の逃げ形成時、逃げ集団へ入る成功率を上げる。</x:v>
       </x:c>
       <x:c r="K151" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="L151" s="38" t="str">
-        <x:v>bikeControl / technique / fighting</x:v>
+        <x:v>stamina / cruise / fighting / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="34" customHeight="1">
@@ -5906,55 +5906,295 @@
       <x:c r="C152" s="38" t="str"/>
       <x:c r="D152" s="38" t="str"/>
       <x:c r="E152" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>逃げ屋</x:v>
       </x:c>
       <x:c r="F152" s="38" t="str">
-        <x:v>basic</x:v>
+        <x:v>specialty</x:v>
       </x:c>
       <x:c r="G152" s="41" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H152" s="41" t="str"/>
       <x:c r="I152" s="38" t="str">
+        <x:v>ブリッジ</x:v>
+      </x:c>
+      <x:c r="J152" s="38" t="str">
+        <x:v>メイン集団から加速し、すでに形成された逃げ集団へ合流する。</x:v>
+      </x:c>
+      <x:c r="K152" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="L152" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="34" customHeight="1">
+      <x:c r="A153" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B153" s="41" t="str"/>
+      <x:c r="C153" s="38" t="str"/>
+      <x:c r="D153" s="38" t="str"/>
+      <x:c r="E153" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F153" s="38" t="str">
+        <x:v>basic</x:v>
+      </x:c>
+      <x:c r="G153" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H153" s="41" t="str"/>
+      <x:c r="I153" s="38" t="str">
+        <x:v>先頭交代</x:v>
+      </x:c>
+      <x:c r="J153" s="38" t="str">
+        <x:v>逃げ集団の先頭を長く引き、本人の体力を使ってタイム差を広げる。</x:v>
+      </x:c>
+      <x:c r="K153" s="38" t="str">
+        <x:v>逃げ集団</x:v>
+      </x:c>
+      <x:c r="L153" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="34" customHeight="1">
+      <x:c r="A154" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B154" s="41" t="str"/>
+      <x:c r="C154" s="38" t="str"/>
+      <x:c r="D154" s="38" t="str"/>
+      <x:c r="E154" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F154" s="38" t="str">
+        <x:v>basic</x:v>
+      </x:c>
+      <x:c r="G154" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H154" s="41" t="str"/>
+      <x:c r="I154" s="38" t="str">
+        <x:v>ペース調整</x:v>
+      </x:c>
+      <x:c r="J154" s="38" t="str">
+        <x:v>余計な体力消費を抑えながら、逃げ集団の速度とタイム差を維持する。</x:v>
+      </x:c>
+      <x:c r="K154" s="38" t="str">
+        <x:v>逃げ集団</x:v>
+      </x:c>
+      <x:c r="L154" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="34" customHeight="1">
+      <x:c r="A155" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B155" s="41" t="str"/>
+      <x:c r="C155" s="38" t="str"/>
+      <x:c r="D155" s="38" t="str"/>
+      <x:c r="E155" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F155" s="38" t="str">
+        <x:v>specialty</x:v>
+      </x:c>
+      <x:c r="G155" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H155" s="41" t="str"/>
+      <x:c r="I155" s="38" t="str">
+        <x:v>逃げ選別</x:v>
+      </x:c>
+      <x:c r="J155" s="38" t="str">
+        <x:v>起伏や横風でペースを上げ、逃げ集団の人数を絞り込む。</x:v>
+      </x:c>
+      <x:c r="K155" s="38" t="str">
+        <x:v>逃げ集団</x:v>
+      </x:c>
+      <x:c r="L155" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="34" customHeight="1">
+      <x:c r="A156" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B156" s="41" t="str"/>
+      <x:c r="C156" s="38" t="str"/>
+      <x:c r="D156" s="38" t="str"/>
+      <x:c r="E156" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F156" s="38" t="str">
+        <x:v>specialty</x:v>
+      </x:c>
+      <x:c r="G156" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H156" s="41" t="str"/>
+      <x:c r="I156" s="38" t="str">
+        <x:v>逃げ粘り</x:v>
+      </x:c>
+      <x:c r="J156" s="38" t="str">
+        <x:v>吸収されそうな場面で再加速し、逃げ集団の生存時間を延ばす。</x:v>
+      </x:c>
+      <x:c r="K156" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="L156" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="34" customHeight="1">
+      <x:c r="A157" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B157" s="41" t="str"/>
+      <x:c r="C157" s="38" t="str"/>
+      <x:c r="D157" s="38" t="str"/>
+      <x:c r="E157" s="38" t="str">
+        <x:v>下り牽引</x:v>
+      </x:c>
+      <x:c r="F157" s="38" t="str">
+        <x:v>basic</x:v>
+      </x:c>
+      <x:c r="G157" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H157" s="41" t="str"/>
+      <x:c r="I157" s="38" t="str">
+        <x:v>高速コーナリング</x:v>
+      </x:c>
+      <x:c r="J157" s="38" t="str">
+        <x:v>コーナーでの速度低下と落車リスクを抑える。</x:v>
+      </x:c>
+      <x:c r="K157" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="L157" s="38" t="str">
+        <x:v>bikeControl / technique / fighting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="34" customHeight="1">
+      <x:c r="A158" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B158" s="41" t="str"/>
+      <x:c r="C158" s="38" t="str"/>
+      <x:c r="D158" s="38" t="str"/>
+      <x:c r="E158" s="38" t="str">
+        <x:v>下り牽引</x:v>
+      </x:c>
+      <x:c r="F158" s="38" t="str">
+        <x:v>specialty</x:v>
+      </x:c>
+      <x:c r="G158" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H158" s="41" t="str"/>
+      <x:c r="I158" s="38" t="str">
+        <x:v>下り加速</x:v>
+      </x:c>
+      <x:c r="J158" s="38" t="str">
+        <x:v>下りの直線で速度を上げ、前方集団との差を縮める。</x:v>
+      </x:c>
+      <x:c r="K158" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="L158" s="38" t="str">
+        <x:v>bikeControl / technique / fighting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="34" customHeight="1">
+      <x:c r="A159" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B159" s="41" t="str"/>
+      <x:c r="C159" s="38" t="str"/>
+      <x:c r="D159" s="38" t="str"/>
+      <x:c r="E159" s="38" t="str">
+        <x:v>下り牽引</x:v>
+      </x:c>
+      <x:c r="F159" s="38" t="str">
+        <x:v>specialty</x:v>
+      </x:c>
+      <x:c r="G159" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H159" s="41" t="str"/>
+      <x:c r="I159" s="38" t="str">
+        <x:v>下りアタック</x:v>
+      </x:c>
+      <x:c r="J159" s="38" t="str">
+        <x:v>テクニカルな下りで仕掛け、後続とのタイム差を作る。</x:v>
+      </x:c>
+      <x:c r="K159" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="L159" s="38" t="str">
+        <x:v>bikeControl / technique / fighting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="34" customHeight="1">
+      <x:c r="A160" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B160" s="41" t="str"/>
+      <x:c r="C160" s="38" t="str"/>
+      <x:c r="D160" s="38" t="str"/>
+      <x:c r="E160" s="38" t="str">
+        <x:v>下り牽引</x:v>
+      </x:c>
+      <x:c r="F160" s="38" t="str">
+        <x:v>basic</x:v>
+      </x:c>
+      <x:c r="G160" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H160" s="41" t="str"/>
+      <x:c r="I160" s="38" t="str">
         <x:v>安全誘導</x:v>
       </x:c>
-      <x:c r="J152" s="38" t="str">
+      <x:c r="J160" s="38" t="str">
         <x:v>安全な走行ラインを示し、味方エースの落車リスクを下げる。</x:v>
       </x:c>
-      <x:c r="K152" s="38" t="str">
-        <x:v>味方エース</x:v>
-      </x:c>
-      <x:c r="L152" s="38" t="str">
+      <x:c r="K160" s="38" t="str">
+        <x:v>味方エース</x:v>
+      </x:c>
+      <x:c r="L160" s="38" t="str">
         <x:v>bikeControl / technique / fighting</x:v>
       </x:c>
     </x:row>
-    <x:row r="153" ht="34" customHeight="1">
-      <x:c r="A153" s="39" t="str">
+    <x:row r="161" ht="34" customHeight="1">
+      <x:c r="A161" s="39" t="str">
         <x:v>役割共通</x:v>
       </x:c>
-      <x:c r="B153" s="42" t="str"/>
-      <x:c r="C153" s="39" t="str"/>
-      <x:c r="D153" s="39" t="str"/>
-      <x:c r="E153" s="39" t="str">
+      <x:c r="B161" s="42" t="str"/>
+      <x:c r="C161" s="39" t="str"/>
+      <x:c r="D161" s="39" t="str"/>
+      <x:c r="E161" s="39" t="str">
         <x:v>下り牽引</x:v>
       </x:c>
-      <x:c r="F153" s="39" t="str">
+      <x:c r="F161" s="39" t="str">
         <x:v>specialty</x:v>
       </x:c>
-      <x:c r="G153" s="42" t="n">
+      <x:c r="G161" s="42" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="H153" s="42" t="str"/>
-      <x:c r="I153" s="39" t="str">
+      <x:c r="H161" s="42" t="str"/>
+      <x:c r="I161" s="39" t="str">
         <x:v>下り復帰</x:v>
       </x:c>
-      <x:c r="J153" s="39" t="str">
+      <x:c r="J161" s="39" t="str">
         <x:v>下りで遅れた味方を牽引し、プロトンや前方集団へ復帰させる。</x:v>
       </x:c>
-      <x:c r="K153" s="39" t="str">
-        <x:v>味方エース</x:v>
-      </x:c>
-      <x:c r="L153" s="39" t="str">
+      <x:c r="K161" s="39" t="str">
+        <x:v>味方エース</x:v>
+      </x:c>
+      <x:c r="L161" s="39" t="str">
         <x:v>bikeControl / technique / fighting</x:v>
       </x:c>
     </x:row>
@@ -5963,14 +6203,14 @@
     <x:mergeCell ref="A1:L1"/>
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="F5:F153">
+  <x:conditionalFormatting sqref="F5:F161">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="basic"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="specialty"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="decisive"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d6053df64d440b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24f0a5008ebf404f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6820,7 +7060,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d8cb501cb584fba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e1d86a533f64b33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6859,7 +7099,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="25" t="str">
-        <x:v>選手固有にしないコスト2の得意技。地形別共通16枚と役割共通18枚の全34枚です。</x:v>
+        <x:v>選手固有にしないコスト2の得意技。地形別共通24枚と役割共通18枚の全42枚です。</x:v>
       </x:c>
       <x:c r="B2" s="25"/>
       <x:c r="C2" s="25"/>
@@ -7023,23 +7263,23 @@
       <x:c r="C9" s="38" t="str"/>
       <x:c r="D9" s="38" t="str"/>
       <x:c r="E9" s="38" t="str">
-        <x:v>丘陵エース</x:v>
+        <x:v>平坦アシスト</x:v>
       </x:c>
       <x:c r="F9" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="41" t="str"/>
       <x:c r="H9" s="47" t="str">
-        <x:v>丘陵加速</x:v>
+        <x:v>位置取り護衛</x:v>
       </x:c>
       <x:c r="I9" s="38" t="str">
-        <x:v>起伏の変化に合わせて加速し、丘陵区間で集団を絞り込む。</x:v>
+        <x:v>混雑した集団内で進路を確保し、味方エースを前方へ引き上げる。</x:v>
       </x:c>
       <x:c r="J9" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K9" s="38" t="str">
-        <x:v>punch / acceleration</x:v>
+        <x:v>positioning / technique / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -7050,23 +7290,23 @@
       <x:c r="C10" s="38" t="str"/>
       <x:c r="D10" s="38" t="str"/>
       <x:c r="E10" s="38" t="str">
-        <x:v>丘陵エース</x:v>
+        <x:v>平坦アシスト</x:v>
       </x:c>
       <x:c r="F10" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G10" s="41" t="str"/>
       <x:c r="H10" s="47" t="str">
-        <x:v>短坂アタック</x:v>
+        <x:v>ローテーション牽引</x:v>
       </x:c>
       <x:c r="I10" s="38" t="str">
-        <x:v>短い急坂で鋭く仕掛け、ライバルとの小さな差を作る。</x:v>
+        <x:v>味方と先頭交代しながら高速巡航を維持し、エースの消耗を抑える。</x:v>
       </x:c>
       <x:c r="J10" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K10" s="38" t="str">
-        <x:v>punch / fighting</x:v>
+        <x:v>cruise / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -7077,23 +7317,23 @@
       <x:c r="C11" s="38" t="str"/>
       <x:c r="D11" s="38" t="str"/>
       <x:c r="E11" s="38" t="str">
-        <x:v>丘陵アシスト</x:v>
+        <x:v>丘陵エース</x:v>
       </x:c>
       <x:c r="F11" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G11" s="41" t="str"/>
       <x:c r="H11" s="47" t="str">
-        <x:v>丘陵ペース</x:v>
+        <x:v>丘陵加速</x:v>
       </x:c>
       <x:c r="I11" s="38" t="str">
-        <x:v>起伏区間を高い一定速度で牽引し、味方エースの脚を残す。</x:v>
+        <x:v>起伏の変化に合わせて加速し、丘陵区間で集団を絞り込む。</x:v>
       </x:c>
       <x:c r="J11" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="K11" s="38" t="str">
-        <x:v>punch / stamina / teamwork</x:v>
+        <x:v>punch / acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
@@ -7104,23 +7344,23 @@
       <x:c r="C12" s="38" t="str"/>
       <x:c r="D12" s="38" t="str"/>
       <x:c r="E12" s="38" t="str">
-        <x:v>丘陵アシスト</x:v>
+        <x:v>丘陵エース</x:v>
       </x:c>
       <x:c r="F12" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G12" s="41" t="str"/>
       <x:c r="H12" s="47" t="str">
-        <x:v>仕掛け封じ</x:v>
+        <x:v>短坂アタック</x:v>
       </x:c>
       <x:c r="I12" s="38" t="str">
-        <x:v>丘陵で危険な攻撃を追走し、味方エースに代わって差を消す。</x:v>
+        <x:v>短い急坂で鋭く仕掛け、ライバルとの小さな差を作る。</x:v>
       </x:c>
       <x:c r="J12" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="K12" s="38" t="str">
-        <x:v>acceleration / fighting / teamwork</x:v>
+        <x:v>punch / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -7131,23 +7371,23 @@
       <x:c r="C13" s="38" t="str"/>
       <x:c r="D13" s="38" t="str"/>
       <x:c r="E13" s="38" t="str">
-        <x:v>山岳エース</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F13" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G13" s="41" t="str"/>
       <x:c r="H13" s="47" t="str">
-        <x:v>登坂ペースアップ</x:v>
+        <x:v>丘陵ペース</x:v>
       </x:c>
       <x:c r="I13" s="38" t="str">
-        <x:v>登りで段階的に速度を上げ、追走できるライバルを絞り込む。</x:v>
+        <x:v>起伏区間を高い一定速度で牽引し、味方エースの脚を残す。</x:v>
       </x:c>
       <x:c r="J13" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K13" s="38" t="str">
-        <x:v>climbing / stamina</x:v>
+        <x:v>punch / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -7158,23 +7398,23 @@
       <x:c r="C14" s="38" t="str"/>
       <x:c r="D14" s="38" t="str"/>
       <x:c r="E14" s="38" t="str">
-        <x:v>山岳エース</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F14" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="41" t="str"/>
       <x:c r="H14" s="47" t="str">
-        <x:v>頂上前加速</x:v>
+        <x:v>仕掛け封じ</x:v>
       </x:c>
       <x:c r="I14" s="38" t="str">
-        <x:v>山頂前で加速し、下りへ入る前に有利な位置と時間差を作る。</x:v>
+        <x:v>丘陵で危険な攻撃を追走し、味方エースに代わって差を消す。</x:v>
       </x:c>
       <x:c r="J14" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K14" s="38" t="str">
-        <x:v>climbing / acceleration</x:v>
+        <x:v>acceleration / fighting / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -7185,23 +7425,23 @@
       <x:c r="C15" s="38" t="str"/>
       <x:c r="D15" s="38" t="str"/>
       <x:c r="E15" s="38" t="str">
-        <x:v>山岳アシスト</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F15" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G15" s="41" t="str"/>
       <x:c r="H15" s="47" t="str">
-        <x:v>山岳先導</x:v>
+        <x:v>坂前誘導</x:v>
       </x:c>
       <x:c r="I15" s="38" t="str">
-        <x:v>山岳終盤まで高いペースで牽引し、味方エースを攻撃位置へ運ぶ。</x:v>
+        <x:v>登りに入る前に味方エースを集団前方へ運び、仕掛けへ備える。</x:v>
       </x:c>
       <x:c r="J15" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K15" s="38" t="str">
-        <x:v>climbing / stamina / teamwork</x:v>
+        <x:v>positioning / acceleration / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -7212,23 +7452,23 @@
       <x:c r="C16" s="38" t="str"/>
       <x:c r="D16" s="38" t="str"/>
       <x:c r="E16" s="38" t="str">
-        <x:v>山岳アシスト</x:v>
+        <x:v>丘陵アシスト</x:v>
       </x:c>
       <x:c r="F16" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G16" s="41" t="str"/>
       <x:c r="H16" s="47" t="str">
-        <x:v>登坂チェイス</x:v>
+        <x:v>丘越え牽引</x:v>
       </x:c>
       <x:c r="I16" s="38" t="str">
-        <x:v>登りで生まれた差を一定ペースで詰め、味方エースを先頭へ戻す。</x:v>
+        <x:v>丘の頂上まで牽引し、味方エースの体力と加速力を温存する。</x:v>
       </x:c>
       <x:c r="J16" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K16" s="38" t="str">
-        <x:v>climbing / recovery / teamwork</x:v>
+        <x:v>punch / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
@@ -7239,23 +7479,23 @@
       <x:c r="C17" s="38" t="str"/>
       <x:c r="D17" s="38" t="str"/>
       <x:c r="E17" s="38" t="str">
-        <x:v>パヴェエース</x:v>
+        <x:v>山岳エース</x:v>
       </x:c>
       <x:c r="F17" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G17" s="41" t="str"/>
       <x:c r="H17" s="47" t="str">
-        <x:v>石畳加速</x:v>
+        <x:v>登坂ペースアップ</x:v>
       </x:c>
       <x:c r="I17" s="38" t="str">
-        <x:v>安定した走行線から加速し、パヴェ区間で先頭位置を奪う。</x:v>
+        <x:v>登りで段階的に速度を上げ、追走できるライバルを絞り込む。</x:v>
       </x:c>
       <x:c r="J17" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="K17" s="38" t="str">
-        <x:v>cobble / acceleration / bike_control</x:v>
+        <x:v>climbing / stamina</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -7266,23 +7506,23 @@
       <x:c r="C18" s="38" t="str"/>
       <x:c r="D18" s="38" t="str"/>
       <x:c r="E18" s="38" t="str">
-        <x:v>パヴェエース</x:v>
+        <x:v>山岳エース</x:v>
       </x:c>
       <x:c r="F18" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G18" s="41" t="str"/>
       <x:c r="H18" s="47" t="str">
-        <x:v>悪路アタック</x:v>
+        <x:v>頂上前加速</x:v>
       </x:c>
       <x:c r="I18" s="38" t="str">
-        <x:v>路面の乱れを利用して仕掛け、悪路に弱いライバルを引き離す。</x:v>
+        <x:v>山頂前で加速し、下りへ入る前に有利な位置と時間差を作る。</x:v>
       </x:c>
       <x:c r="J18" s="38" t="str">
         <x:v>本人</x:v>
       </x:c>
       <x:c r="K18" s="38" t="str">
-        <x:v>cobble / fighting</x:v>
+        <x:v>climbing / acceleration</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
@@ -7293,23 +7533,23 @@
       <x:c r="C19" s="38" t="str"/>
       <x:c r="D19" s="38" t="str"/>
       <x:c r="E19" s="38" t="str">
-        <x:v>パヴェアシスト</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F19" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G19" s="41" t="str"/>
       <x:c r="H19" s="47" t="str">
-        <x:v>石畳牽引</x:v>
+        <x:v>山岳先導</x:v>
       </x:c>
       <x:c r="I19" s="38" t="str">
-        <x:v>悪路で安全な走行線を保ちながら牽引し、味方エースを前方へ運ぶ。</x:v>
+        <x:v>山岳終盤まで高いペースで牽引し、味方エースを攻撃位置へ運ぶ。</x:v>
       </x:c>
       <x:c r="J19" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K19" s="38" t="str">
-        <x:v>cobble / bike_control / teamwork</x:v>
+        <x:v>climbing / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
@@ -7320,239 +7560,239 @@
       <x:c r="C20" s="38" t="str"/>
       <x:c r="D20" s="38" t="str"/>
       <x:c r="E20" s="38" t="str">
-        <x:v>パヴェアシスト</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F20" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G20" s="41" t="str"/>
       <x:c r="H20" s="47" t="str">
-        <x:v>パヴェ追走</x:v>
+        <x:v>登坂チェイス</x:v>
       </x:c>
       <x:c r="I20" s="38" t="str">
-        <x:v>パヴェで先行した危険な選手を追い、味方エースを先頭集団へ戻す。</x:v>
+        <x:v>登りで生まれた差を一定ペースで詰め、味方エースを先頭へ戻す。</x:v>
       </x:c>
       <x:c r="J20" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K20" s="38" t="str">
-        <x:v>cobble / cruise / teamwork</x:v>
+        <x:v>climbing / recovery / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
       <x:c r="A21" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B21" s="41" t="str"/>
       <x:c r="C21" s="38" t="str"/>
       <x:c r="D21" s="38" t="str"/>
       <x:c r="E21" s="38" t="str">
-        <x:v>サブエース</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F21" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G21" s="41" t="str"/>
       <x:c r="H21" s="47" t="str">
-        <x:v>プランB</x:v>
+        <x:v>登り口誘導</x:v>
       </x:c>
       <x:c r="I21" s="38" t="str">
-        <x:v>エースの不調や脱落時に第二の勝利プランへ移行する。</x:v>
+        <x:v>山岳開始前に集団前方を確保し、味方エースを安全に登りへ入れる。</x:v>
       </x:c>
       <x:c r="J21" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K21" s="38" t="str">
-        <x:v>ace_aptitude / recovery / fighting</x:v>
+        <x:v>positioning / climbing / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
       <x:c r="A22" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B22" s="41" t="str"/>
       <x:c r="C22" s="38" t="str"/>
       <x:c r="D22" s="38" t="str"/>
       <x:c r="E22" s="38" t="str">
-        <x:v>ロードキャプテン</x:v>
+        <x:v>山岳アシスト</x:v>
       </x:c>
       <x:c r="F22" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G22" s="41" t="str"/>
       <x:c r="H22" s="47" t="str">
-        <x:v>隊列再編</x:v>
+        <x:v>山岳風よけ</x:v>
       </x:c>
       <x:c r="I22" s="38" t="str">
-        <x:v>味方の位置取りと戦術判断を安定させる。</x:v>
+        <x:v>登りで風よけとなり、味方エースの体力消費を抑える。</x:v>
       </x:c>
       <x:c r="J22" s="38" t="str">
-        <x:v>味方チーム</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K22" s="38" t="str">
-        <x:v>teamwork / technique / recovery</x:v>
+        <x:v>climbing / stamina / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
       <x:c r="A23" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B23" s="41" t="str"/>
       <x:c r="C23" s="38" t="str"/>
       <x:c r="D23" s="38" t="str"/>
       <x:c r="E23" s="38" t="str">
-        <x:v>リードアウト</x:v>
+        <x:v>パヴェエース</x:v>
       </x:c>
       <x:c r="F23" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G23" s="41" t="str"/>
       <x:c r="H23" s="47" t="str">
-        <x:v>高速リードアウト</x:v>
+        <x:v>石畳加速</x:v>
       </x:c>
       <x:c r="I23" s="38" t="str">
-        <x:v>味方スプリンターの位置取りと加速移行を補助する。</x:v>
+        <x:v>安定した走行線から加速し、パヴェ区間で先頭位置を奪う。</x:v>
       </x:c>
       <x:c r="J23" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="K23" s="38" t="str">
-        <x:v>acceleration / sprint / cruise / teamwork</x:v>
+        <x:v>cobble / acceleration / bike_control</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
       <x:c r="A24" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B24" s="41" t="str"/>
       <x:c r="C24" s="38" t="str"/>
       <x:c r="D24" s="38" t="str"/>
       <x:c r="E24" s="38" t="str">
-        <x:v>スプリントトレイン</x:v>
+        <x:v>パヴェエース</x:v>
       </x:c>
       <x:c r="F24" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G24" s="41" t="str"/>
       <x:c r="H24" s="47" t="str">
-        <x:v>トレイン加速</x:v>
+        <x:v>悪路アタック</x:v>
       </x:c>
       <x:c r="I24" s="38" t="str">
-        <x:v>終盤の隊列維持と速度の受け渡しを安定させる。</x:v>
+        <x:v>路面の乱れを利用して仕掛け、悪路に弱いライバルを引き離す。</x:v>
       </x:c>
       <x:c r="J24" s="38" t="str">
-        <x:v>味方チーム</x:v>
+        <x:v>本人</x:v>
       </x:c>
       <x:c r="K24" s="38" t="str">
-        <x:v>cruise / acceleration / sprint / teamwork</x:v>
+        <x:v>cobble / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
       <x:c r="A25" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B25" s="41" t="str"/>
       <x:c r="C25" s="38" t="str"/>
       <x:c r="D25" s="38" t="str"/>
       <x:c r="E25" s="38" t="str">
-        <x:v>平坦ペースメーカー</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F25" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="41" t="str"/>
       <x:c r="H25" s="47" t="str">
-        <x:v>ハイペース維持</x:v>
+        <x:v>石畳牽引</x:v>
       </x:c>
       <x:c r="I25" s="38" t="str">
-        <x:v>逃げとの差と集団速度を安定させる。</x:v>
+        <x:v>悪路で安全な走行線を保ちながら牽引し、味方エースを前方へ運ぶ。</x:v>
       </x:c>
       <x:c r="J25" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K25" s="38" t="str">
-        <x:v>cruise / stamina / recovery</x:v>
+        <x:v>cobble / bike_control / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
       <x:c r="A26" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B26" s="41" t="str"/>
       <x:c r="C26" s="38" t="str"/>
       <x:c r="D26" s="38" t="str"/>
       <x:c r="E26" s="38" t="str">
-        <x:v>山岳番手</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F26" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G26" s="41" t="str"/>
       <x:c r="H26" s="47" t="str">
-        <x:v>最後の山岳牽引</x:v>
+        <x:v>パヴェ追走</x:v>
       </x:c>
       <x:c r="I26" s="38" t="str">
-        <x:v>山頂付近の攻撃対応と最終発射を支援する。</x:v>
+        <x:v>パヴェで先行した危険な選手を追い、味方エースを先頭集団へ戻す。</x:v>
       </x:c>
       <x:c r="J26" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K26" s="38" t="str">
-        <x:v>climb / acceleration / stamina / recovery</x:v>
+        <x:v>cobble / cruise / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="34" customHeight="1">
       <x:c r="A27" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B27" s="41" t="str"/>
       <x:c r="C27" s="38" t="str"/>
       <x:c r="D27" s="38" t="str"/>
       <x:c r="E27" s="38" t="str">
-        <x:v>山岳ペースメーカー</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F27" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G27" s="41" t="str"/>
       <x:c r="H27" s="47" t="str">
-        <x:v>山岳ペースアップ</x:v>
+        <x:v>石畳進入</x:v>
       </x:c>
       <x:c r="I27" s="38" t="str">
-        <x:v>集団を絞り込み急なアタックを抑制する。</x:v>
+        <x:v>パヴェ区間へ入る前に前方位置を確保し、分断や落車の危険を抑える。</x:v>
       </x:c>
       <x:c r="J27" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K27" s="38" t="str">
-        <x:v>climb / stamina / cruise</x:v>
+        <x:v>positioning / cobble / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="34" customHeight="1">
       <x:c r="A28" s="38" t="str">
-        <x:v>役割共通</x:v>
+        <x:v>共通得意技</x:v>
       </x:c>
       <x:c r="B28" s="41" t="str"/>
       <x:c r="C28" s="38" t="str"/>
       <x:c r="D28" s="38" t="str"/>
       <x:c r="E28" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>パヴェアシスト</x:v>
       </x:c>
       <x:c r="F28" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="41" t="str"/>
       <x:c r="H28" s="47" t="str">
-        <x:v>ダウンヒル牽引</x:v>
+        <x:v>ライン誘導</x:v>
       </x:c>
       <x:c r="I28" s="38" t="str">
-        <x:v>下り速度と隊列安定性を高める。</x:v>
+        <x:v>石畳で走りやすいラインを示し、味方エースの減速とトラブルを抑える。</x:v>
       </x:c>
       <x:c r="J28" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K28" s="38" t="str">
-        <x:v>bikeControl / technique / fighting</x:v>
+        <x:v>cobble / bike_control / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
@@ -7563,23 +7803,23 @@
       <x:c r="C29" s="38" t="str"/>
       <x:c r="D29" s="38" t="str"/>
       <x:c r="E29" s="38" t="str">
-        <x:v>ブレイクアウェイキラー</x:v>
+        <x:v>サブエース</x:v>
       </x:c>
       <x:c r="F29" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G29" s="41" t="str"/>
       <x:c r="H29" s="47" t="str">
-        <x:v>逃げ吸収</x:v>
+        <x:v>プランB</x:v>
       </x:c>
       <x:c r="I29" s="38" t="str">
-        <x:v>逃げとのタイム差を効率よく削る。</x:v>
+        <x:v>エースの不調や脱落時に第二の勝利プランへ移行する。</x:v>
       </x:c>
       <x:c r="J29" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K29" s="38" t="str">
-        <x:v>cruise / stamina / teamwork</x:v>
+        <x:v>ace_aptitude / recovery / fighting</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
@@ -7590,23 +7830,23 @@
       <x:c r="C30" s="38" t="str"/>
       <x:c r="D30" s="38" t="str"/>
       <x:c r="E30" s="38" t="str">
-        <x:v>トラブル復帰牽引</x:v>
+        <x:v>ロードキャプテン</x:v>
       </x:c>
       <x:c r="F30" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="41" t="str"/>
       <x:c r="H30" s="47" t="str">
-        <x:v>集団復帰</x:v>
+        <x:v>隊列再編</x:v>
       </x:c>
       <x:c r="I30" s="38" t="str">
-        <x:v>復帰速度を上げエースの消耗を抑える。</x:v>
+        <x:v>味方の位置取りと戦術判断を安定させる。</x:v>
       </x:c>
       <x:c r="J30" s="38" t="str">
-        <x:v>味方エース</x:v>
+        <x:v>味方チーム</x:v>
       </x:c>
       <x:c r="K30" s="38" t="str">
-        <x:v>cruise / stamina / teamwork</x:v>
+        <x:v>teamwork / technique / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
@@ -7617,23 +7857,23 @@
       <x:c r="C31" s="38" t="str"/>
       <x:c r="D31" s="38" t="str"/>
       <x:c r="E31" s="38" t="str">
-        <x:v>サテライトライダー</x:v>
+        <x:v>リードアウト</x:v>
       </x:c>
       <x:c r="F31" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G31" s="41" t="str"/>
       <x:c r="H31" s="47" t="str">
-        <x:v>サテライト合流</x:v>
+        <x:v>高速リードアウト</x:v>
       </x:c>
       <x:c r="I31" s="38" t="str">
-        <x:v>合流後に補給、牽引、風よけを提供する。</x:v>
+        <x:v>味方スプリンターの位置取りと加速移行を補助する。</x:v>
       </x:c>
       <x:c r="J31" s="38" t="str">
         <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K31" s="38" t="str">
-        <x:v>climb / stamina / recovery / teamwork</x:v>
+        <x:v>acceleration / sprint / cruise / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
@@ -7644,23 +7884,23 @@
       <x:c r="C32" s="38" t="str"/>
       <x:c r="D32" s="38" t="str"/>
       <x:c r="E32" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>スプリントトレイン</x:v>
       </x:c>
       <x:c r="F32" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G32" s="41" t="str"/>
       <x:c r="H32" s="47" t="str">
-        <x:v>逃げ参加</x:v>
+        <x:v>トレイン加速</x:v>
       </x:c>
       <x:c r="I32" s="38" t="str">
-        <x:v>序盤の逃げ形成時、逃げ集団へ入る成功率を上げる。</x:v>
+        <x:v>終盤の隊列維持と速度の受け渡しを安定させる。</x:v>
       </x:c>
       <x:c r="J32" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方チーム</x:v>
       </x:c>
       <x:c r="K32" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>cruise / acceleration / sprint / teamwork</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
@@ -7671,23 +7911,23 @@
       <x:c r="C33" s="38" t="str"/>
       <x:c r="D33" s="38" t="str"/>
       <x:c r="E33" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>平坦ペースメーカー</x:v>
       </x:c>
       <x:c r="F33" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G33" s="41" t="str"/>
       <x:c r="H33" s="47" t="str">
-        <x:v>ブリッジ</x:v>
+        <x:v>ハイペース維持</x:v>
       </x:c>
       <x:c r="I33" s="38" t="str">
-        <x:v>メイン集団から加速し、すでに形成された逃げ集団へ合流する。</x:v>
+        <x:v>逃げとの差と集団速度を安定させる。</x:v>
       </x:c>
       <x:c r="J33" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K33" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>cruise / stamina / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
@@ -7698,23 +7938,23 @@
       <x:c r="C34" s="38" t="str"/>
       <x:c r="D34" s="38" t="str"/>
       <x:c r="E34" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>山岳番手</x:v>
       </x:c>
       <x:c r="F34" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G34" s="41" t="str"/>
       <x:c r="H34" s="47" t="str">
-        <x:v>逃げ選別</x:v>
+        <x:v>最後の山岳牽引</x:v>
       </x:c>
       <x:c r="I34" s="38" t="str">
-        <x:v>起伏や横風でペースを上げ、逃げ集団の人数を絞り込む。</x:v>
+        <x:v>山頂付近の攻撃対応と最終発射を支援する。</x:v>
       </x:c>
       <x:c r="J34" s="38" t="str">
-        <x:v>逃げ集団</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K34" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>climb / acceleration / stamina / recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
@@ -7725,23 +7965,23 @@
       <x:c r="C35" s="38" t="str"/>
       <x:c r="D35" s="38" t="str"/>
       <x:c r="E35" s="38" t="str">
-        <x:v>逃げ屋</x:v>
+        <x:v>山岳ペースメーカー</x:v>
       </x:c>
       <x:c r="F35" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G35" s="41" t="str"/>
       <x:c r="H35" s="47" t="str">
-        <x:v>逃げ粘り</x:v>
+        <x:v>山岳ペースアップ</x:v>
       </x:c>
       <x:c r="I35" s="38" t="str">
-        <x:v>吸収されそうな場面で再加速し、逃げ集団の生存時間を延ばす。</x:v>
+        <x:v>集団を絞り込み急なアタックを抑制する。</x:v>
       </x:c>
       <x:c r="J35" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K35" s="38" t="str">
-        <x:v>stamina / cruise / fighting / recovery</x:v>
+        <x:v>climb / stamina / cruise</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
@@ -7759,13 +7999,13 @@
       </x:c>
       <x:c r="G36" s="41" t="str"/>
       <x:c r="H36" s="47" t="str">
-        <x:v>下り加速</x:v>
+        <x:v>ダウンヒル牽引</x:v>
       </x:c>
       <x:c r="I36" s="38" t="str">
-        <x:v>下りの直線で速度を上げ、前方集団との差を縮める。</x:v>
+        <x:v>下り速度と隊列安定性を高める。</x:v>
       </x:c>
       <x:c r="J36" s="38" t="str">
-        <x:v>本人</x:v>
+        <x:v>味方エース</x:v>
       </x:c>
       <x:c r="K36" s="38" t="str">
         <x:v>bikeControl / technique / fighting</x:v>
@@ -7779,49 +8019,265 @@
       <x:c r="C37" s="38" t="str"/>
       <x:c r="D37" s="38" t="str"/>
       <x:c r="E37" s="38" t="str">
-        <x:v>下り牽引</x:v>
+        <x:v>ブレイクアウェイキラー</x:v>
       </x:c>
       <x:c r="F37" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G37" s="41" t="str"/>
       <x:c r="H37" s="47" t="str">
+        <x:v>逃げ吸収</x:v>
+      </x:c>
+      <x:c r="I37" s="38" t="str">
+        <x:v>逃げとのタイム差を効率よく削る。</x:v>
+      </x:c>
+      <x:c r="J37" s="38" t="str">
+        <x:v>味方エース</x:v>
+      </x:c>
+      <x:c r="K37" s="38" t="str">
+        <x:v>cruise / stamina / teamwork</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B38" s="41" t="str"/>
+      <x:c r="C38" s="38" t="str"/>
+      <x:c r="D38" s="38" t="str"/>
+      <x:c r="E38" s="38" t="str">
+        <x:v>トラブル復帰牽引</x:v>
+      </x:c>
+      <x:c r="F38" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G38" s="41" t="str"/>
+      <x:c r="H38" s="47" t="str">
+        <x:v>集団復帰</x:v>
+      </x:c>
+      <x:c r="I38" s="38" t="str">
+        <x:v>復帰速度を上げエースの消耗を抑える。</x:v>
+      </x:c>
+      <x:c r="J38" s="38" t="str">
+        <x:v>味方エース</x:v>
+      </x:c>
+      <x:c r="K38" s="38" t="str">
+        <x:v>cruise / stamina / teamwork</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="34" customHeight="1">
+      <x:c r="A39" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B39" s="41" t="str"/>
+      <x:c r="C39" s="38" t="str"/>
+      <x:c r="D39" s="38" t="str"/>
+      <x:c r="E39" s="38" t="str">
+        <x:v>サテライトライダー</x:v>
+      </x:c>
+      <x:c r="F39" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G39" s="41" t="str"/>
+      <x:c r="H39" s="47" t="str">
+        <x:v>サテライト合流</x:v>
+      </x:c>
+      <x:c r="I39" s="38" t="str">
+        <x:v>合流後に補給、牽引、風よけを提供する。</x:v>
+      </x:c>
+      <x:c r="J39" s="38" t="str">
+        <x:v>味方エース</x:v>
+      </x:c>
+      <x:c r="K39" s="38" t="str">
+        <x:v>climb / stamina / recovery / teamwork</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B40" s="41" t="str"/>
+      <x:c r="C40" s="38" t="str"/>
+      <x:c r="D40" s="38" t="str"/>
+      <x:c r="E40" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F40" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G40" s="41" t="str"/>
+      <x:c r="H40" s="47" t="str">
+        <x:v>逃げ参加</x:v>
+      </x:c>
+      <x:c r="I40" s="38" t="str">
+        <x:v>序盤の逃げ形成時、逃げ集団へ入る成功率を上げる。</x:v>
+      </x:c>
+      <x:c r="J40" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="K40" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B41" s="41" t="str"/>
+      <x:c r="C41" s="38" t="str"/>
+      <x:c r="D41" s="38" t="str"/>
+      <x:c r="E41" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F41" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G41" s="41" t="str"/>
+      <x:c r="H41" s="47" t="str">
+        <x:v>ブリッジ</x:v>
+      </x:c>
+      <x:c r="I41" s="38" t="str">
+        <x:v>メイン集団から加速し、すでに形成された逃げ集団へ合流する。</x:v>
+      </x:c>
+      <x:c r="J41" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="K41" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B42" s="41" t="str"/>
+      <x:c r="C42" s="38" t="str"/>
+      <x:c r="D42" s="38" t="str"/>
+      <x:c r="E42" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F42" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G42" s="41" t="str"/>
+      <x:c r="H42" s="47" t="str">
+        <x:v>逃げ選別</x:v>
+      </x:c>
+      <x:c r="I42" s="38" t="str">
+        <x:v>起伏や横風でペースを上げ、逃げ集団の人数を絞り込む。</x:v>
+      </x:c>
+      <x:c r="J42" s="38" t="str">
+        <x:v>逃げ集団</x:v>
+      </x:c>
+      <x:c r="K42" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B43" s="41" t="str"/>
+      <x:c r="C43" s="38" t="str"/>
+      <x:c r="D43" s="38" t="str"/>
+      <x:c r="E43" s="38" t="str">
+        <x:v>逃げ屋</x:v>
+      </x:c>
+      <x:c r="F43" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G43" s="41" t="str"/>
+      <x:c r="H43" s="47" t="str">
+        <x:v>逃げ粘り</x:v>
+      </x:c>
+      <x:c r="I43" s="38" t="str">
+        <x:v>吸収されそうな場面で再加速し、逃げ集団の生存時間を延ばす。</x:v>
+      </x:c>
+      <x:c r="J43" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="K43" s="38" t="str">
+        <x:v>stamina / cruise / fighting / recovery</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B44" s="41" t="str"/>
+      <x:c r="C44" s="38" t="str"/>
+      <x:c r="D44" s="38" t="str"/>
+      <x:c r="E44" s="38" t="str">
+        <x:v>下り牽引</x:v>
+      </x:c>
+      <x:c r="F44" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G44" s="41" t="str"/>
+      <x:c r="H44" s="47" t="str">
+        <x:v>下り加速</x:v>
+      </x:c>
+      <x:c r="I44" s="38" t="str">
+        <x:v>下りの直線で速度を上げ、前方集団との差を縮める。</x:v>
+      </x:c>
+      <x:c r="J44" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="K44" s="38" t="str">
+        <x:v>bikeControl / technique / fighting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="38" t="str">
+        <x:v>役割共通</x:v>
+      </x:c>
+      <x:c r="B45" s="41" t="str"/>
+      <x:c r="C45" s="38" t="str"/>
+      <x:c r="D45" s="38" t="str"/>
+      <x:c r="E45" s="38" t="str">
+        <x:v>下り牽引</x:v>
+      </x:c>
+      <x:c r="F45" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G45" s="41" t="str"/>
+      <x:c r="H45" s="47" t="str">
         <x:v>下りアタック</x:v>
       </x:c>
-      <x:c r="I37" s="38" t="str">
+      <x:c r="I45" s="38" t="str">
         <x:v>テクニカルな下りで仕掛け、後続とのタイム差を作る。</x:v>
       </x:c>
-      <x:c r="J37" s="38" t="str">
-        <x:v>本人</x:v>
-      </x:c>
-      <x:c r="K37" s="38" t="str">
+      <x:c r="J45" s="38" t="str">
+        <x:v>本人</x:v>
+      </x:c>
+      <x:c r="K45" s="38" t="str">
         <x:v>bikeControl / technique / fighting</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="34" customHeight="1">
-      <x:c r="A38" s="39" t="str">
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="39" t="str">
         <x:v>役割共通</x:v>
       </x:c>
-      <x:c r="B38" s="42" t="str"/>
-      <x:c r="C38" s="39" t="str"/>
-      <x:c r="D38" s="39" t="str"/>
-      <x:c r="E38" s="39" t="str">
+      <x:c r="B46" s="42" t="str"/>
+      <x:c r="C46" s="39" t="str"/>
+      <x:c r="D46" s="39" t="str"/>
+      <x:c r="E46" s="39" t="str">
         <x:v>下り牽引</x:v>
       </x:c>
-      <x:c r="F38" s="42" t="n">
+      <x:c r="F46" s="42" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G38" s="42" t="str"/>
-      <x:c r="H38" s="48" t="str">
+      <x:c r="G46" s="42" t="str"/>
+      <x:c r="H46" s="48" t="str">
         <x:v>下り復帰</x:v>
       </x:c>
-      <x:c r="I38" s="39" t="str">
+      <x:c r="I46" s="39" t="str">
         <x:v>下りで遅れた味方を牽引し、プロトンや前方集団へ復帰させる。</x:v>
       </x:c>
-      <x:c r="J38" s="39" t="str">
-        <x:v>味方エース</x:v>
-      </x:c>
-      <x:c r="K38" s="39" t="str">
+      <x:c r="J46" s="39" t="str">
+        <x:v>味方エース</x:v>
+      </x:c>
+      <x:c r="K46" s="39" t="str">
         <x:v>bikeControl / technique / fighting</x:v>
       </x:c>
     </x:row>
@@ -7832,7 +8288,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd77b3873b1344731"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e58aa573edf4a9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8610,7 +9066,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R867fefb08d6441ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86ae607dde354973"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10454,7 +10910,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ad1ad3199041fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65e415620dd24dee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11027,7 +11483,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61c6e68a8c894e95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68824d9f19c2494c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11680,7 +12136,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22b8ccee325e49f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf964166baea4514"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11845,10 +12301,10 @@
         <x:v>得意技の共通テンプレート</x:v>
       </x:c>
       <x:c r="C13" s="41" t="n">
-        <x:v>16</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D13" s="38" t="str">
-        <x:v>4地形×2役割×各2枚</x:v>
+        <x:v>4地形×（エース2枚＋アシスト4枚）</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -11928,7 +12384,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42e329778ed74e8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08135afc11714379"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>